<commit_message>
Correct distortion naming and curve example
Co-authored-by: Higanbana-TW <Higanbana-TW@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lens_distortion_line_calculator.xlsx
+++ b/lens_distortion_line_calculator.xlsx
@@ -745,7 +745,7 @@
         <v>-100</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>-50</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -771,7 +771,7 @@
         <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>本檔使用 Distortion(%)=(畸變像高/理想像高-1)×100%。正值是 barrel 方向的向外位移，負值是 pincushion 方向的向內位移。若鏡頭資料表使用相反符號或 TV distortion，需先轉換，不能直接套用。</t>
+          <t>本檔使用 Distortion(%)=(畸變像高/理想像高-1)×100%。正值是向外位移（通常稱 pincushion），負值是向內位移（通常稱 barrel）。若鏡頭資料表使用相反符號或 TV distortion，需先轉換，不能直接套用。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use consistent LUT interpolation for verification
Co-authored-by: Higanbana-TW <Higanbana-TW@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lens_distortion_line_calculator.xlsx
+++ b/lens_distortion_line_calculator.xlsx
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="E13" s="8">
-        <f>IF(E12&lt;2,"錯誤：至少 2 列",IF(COUNTBLANK(A19:INDEX(A:A,18+E12))+COUNTBLANK(B19:INDEX(B:B,18+E12))&gt;0,"錯誤：中間不可空白",IF(SUMPRODUCT(--(A20:INDEX(A:A,18+E12)&lt;=A19:INDEX(A:A,17+E12)))&gt;0,"錯誤：半視角須遞增",IF(SUMPRODUCT(--(D20:INDEX(D:D,18+E12)&lt;=D19:INDEX(D:D,17+E12)))&gt;0,"錯誤：畸變像高須遞增","OK"))))</f>
+        <f>IF(E12&lt;2,"錯誤：至少 2 列",IF(A19&lt;&gt;0,"錯誤：首列半視角須為 0",IF(COUNTBLANK(A19:INDEX(A:A,18+E12))+COUNTBLANK(B19:INDEX(B:B,18+E12))&gt;0,"錯誤：中間不可空白",IF(SUMPRODUCT(--(A20:INDEX(A:A,18+E12)&lt;=A19:INDEX(A:A,17+E12)))&gt;0,"錯誤：半視角須遞增",IF(SUMPRODUCT(--(D20:INDEX(D:D,18+E12)&lt;=D19:INDEX(D:D,17+E12)))&gt;0,"錯誤：畸變像高須遞增","OK")))))</f>
         <v/>
       </c>
     </row>
@@ -1296,11 +1296,11 @@
         <v/>
       </c>
       <c r="X19">
-        <f>IF(OR($E$13&lt;&gt;"OK",M19=""),"",IF(M19&lt;=$A$19,$B$19,IF(M19&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M19-INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M19=""),"",IF(M19&lt;=$A$19,$D$19,IF(M19&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M19-INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M19,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y19">
-        <f>IF(M19="","",$B$5*TAN(RADIANS(M19))*(1+X19/100)*1000/$B$4)</f>
+        <f>IF(X19="","",X19*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1385,11 +1385,11 @@
         <v/>
       </c>
       <c r="X20">
-        <f>IF(OR($E$13&lt;&gt;"OK",M20=""),"",IF(M20&lt;=$A$19,$B$19,IF(M20&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M20-INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M20=""),"",IF(M20&lt;=$A$19,$D$19,IF(M20&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M20-INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M20,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y20">
-        <f>IF(M20="","",$B$5*TAN(RADIANS(M20))*(1+X20/100)*1000/$B$4)</f>
+        <f>IF(X20="","",X20*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1474,11 +1474,11 @@
         <v/>
       </c>
       <c r="X21">
-        <f>IF(OR($E$13&lt;&gt;"OK",M21=""),"",IF(M21&lt;=$A$19,$B$19,IF(M21&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M21-INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M21=""),"",IF(M21&lt;=$A$19,$D$19,IF(M21&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M21-INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M21,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y21">
-        <f>IF(M21="","",$B$5*TAN(RADIANS(M21))*(1+X21/100)*1000/$B$4)</f>
+        <f>IF(X21="","",X21*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1563,11 +1563,11 @@
         <v/>
       </c>
       <c r="X22">
-        <f>IF(OR($E$13&lt;&gt;"OK",M22=""),"",IF(M22&lt;=$A$19,$B$19,IF(M22&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M22-INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M22=""),"",IF(M22&lt;=$A$19,$D$19,IF(M22&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M22-INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M22,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y22">
-        <f>IF(M22="","",$B$5*TAN(RADIANS(M22))*(1+X22/100)*1000/$B$4)</f>
+        <f>IF(X22="","",X22*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1805,11 +1805,11 @@
         <v/>
       </c>
       <c r="X27">
-        <f>IF(OR($E$13&lt;&gt;"OK",M27=""),"",IF(M27&lt;=$A$19,$B$19,IF(M27&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M27-INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M27=""),"",IF(M27&lt;=$A$19,$D$19,IF(M27&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M27-INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M27,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y27">
-        <f>IF(M27="","",$B$5*TAN(RADIANS(M27))*(1+X27/100)*1000/$B$4)</f>
+        <f>IF(X27="","",X27*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1897,11 +1897,11 @@
         <v/>
       </c>
       <c r="X28">
-        <f>IF(OR($E$13&lt;&gt;"OK",M28=""),"",IF(M28&lt;=$A$19,$B$19,IF(M28&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M28-INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M28=""),"",IF(M28&lt;=$A$19,$D$19,IF(M28&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M28-INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M28,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y28">
-        <f>IF(M28="","",$B$5*TAN(RADIANS(M28))*(1+X28/100)*1000/$B$4)</f>
+        <f>IF(X28="","",X28*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -1989,11 +1989,11 @@
         <v/>
       </c>
       <c r="X29">
-        <f>IF(OR($E$13&lt;&gt;"OK",M29=""),"",IF(M29&lt;=$A$19,$B$19,IF(M29&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M29-INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M29=""),"",IF(M29&lt;=$A$19,$D$19,IF(M29&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M29-INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M29,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y29">
-        <f>IF(M29="","",$B$5*TAN(RADIANS(M29))*(1+X29/100)*1000/$B$4)</f>
+        <f>IF(X29="","",X29*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2081,11 +2081,11 @@
         <v/>
       </c>
       <c r="X30">
-        <f>IF(OR($E$13&lt;&gt;"OK",M30=""),"",IF(M30&lt;=$A$19,$B$19,IF(M30&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M30-INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M30=""),"",IF(M30&lt;=$A$19,$D$19,IF(M30&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M30-INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M30,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y30">
-        <f>IF(M30="","",$B$5*TAN(RADIANS(M30))*(1+X30/100)*1000/$B$4)</f>
+        <f>IF(X30="","",X30*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2173,11 +2173,11 @@
         <v/>
       </c>
       <c r="X31">
-        <f>IF(OR($E$13&lt;&gt;"OK",M31=""),"",IF(M31&lt;=$A$19,$B$19,IF(M31&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M31-INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M31=""),"",IF(M31&lt;=$A$19,$D$19,IF(M31&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M31-INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M31,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y31">
-        <f>IF(M31="","",$B$5*TAN(RADIANS(M31))*(1+X31/100)*1000/$B$4)</f>
+        <f>IF(X31="","",X31*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2265,11 +2265,11 @@
         <v/>
       </c>
       <c r="X32">
-        <f>IF(OR($E$13&lt;&gt;"OK",M32=""),"",IF(M32&lt;=$A$19,$B$19,IF(M32&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M32-INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M32=""),"",IF(M32&lt;=$A$19,$D$19,IF(M32&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M32-INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M32,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y32">
-        <f>IF(M32="","",$B$5*TAN(RADIANS(M32))*(1+X32/100)*1000/$B$4)</f>
+        <f>IF(X32="","",X32*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2357,11 +2357,11 @@
         <v/>
       </c>
       <c r="X33">
-        <f>IF(OR($E$13&lt;&gt;"OK",M33=""),"",IF(M33&lt;=$A$19,$B$19,IF(M33&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M33-INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M33=""),"",IF(M33&lt;=$A$19,$D$19,IF(M33&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M33-INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M33,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y33">
-        <f>IF(M33="","",$B$5*TAN(RADIANS(M33))*(1+X33/100)*1000/$B$4)</f>
+        <f>IF(X33="","",X33*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2449,11 +2449,11 @@
         <v/>
       </c>
       <c r="X34">
-        <f>IF(OR($E$13&lt;&gt;"OK",M34=""),"",IF(M34&lt;=$A$19,$B$19,IF(M34&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M34-INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M34=""),"",IF(M34&lt;=$A$19,$D$19,IF(M34&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M34-INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M34,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y34">
-        <f>IF(M34="","",$B$5*TAN(RADIANS(M34))*(1+X34/100)*1000/$B$4)</f>
+        <f>IF(X34="","",X34*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2541,11 +2541,11 @@
         <v/>
       </c>
       <c r="X35">
-        <f>IF(OR($E$13&lt;&gt;"OK",M35=""),"",IF(M35&lt;=$A$19,$B$19,IF(M35&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M35-INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M35=""),"",IF(M35&lt;=$A$19,$D$19,IF(M35&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M35-INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M35,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y35">
-        <f>IF(M35="","",$B$5*TAN(RADIANS(M35))*(1+X35/100)*1000/$B$4)</f>
+        <f>IF(X35="","",X35*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2633,11 +2633,11 @@
         <v/>
       </c>
       <c r="X36">
-        <f>IF(OR($E$13&lt;&gt;"OK",M36=""),"",IF(M36&lt;=$A$19,$B$19,IF(M36&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M36-INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M36=""),"",IF(M36&lt;=$A$19,$D$19,IF(M36&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M36-INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M36,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y36">
-        <f>IF(M36="","",$B$5*TAN(RADIANS(M36))*(1+X36/100)*1000/$B$4)</f>
+        <f>IF(X36="","",X36*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2725,11 +2725,11 @@
         <v/>
       </c>
       <c r="X37">
-        <f>IF(OR($E$13&lt;&gt;"OK",M37=""),"",IF(M37&lt;=$A$19,$B$19,IF(M37&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M37-INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M37=""),"",IF(M37&lt;=$A$19,$D$19,IF(M37&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M37-INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M37,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y37">
-        <f>IF(M37="","",$B$5*TAN(RADIANS(M37))*(1+X37/100)*1000/$B$4)</f>
+        <f>IF(X37="","",X37*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2817,11 +2817,11 @@
         <v/>
       </c>
       <c r="X38">
-        <f>IF(OR($E$13&lt;&gt;"OK",M38=""),"",IF(M38&lt;=$A$19,$B$19,IF(M38&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M38-INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M38=""),"",IF(M38&lt;=$A$19,$D$19,IF(M38&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M38-INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M38,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y38">
-        <f>IF(M38="","",$B$5*TAN(RADIANS(M38))*(1+X38/100)*1000/$B$4)</f>
+        <f>IF(X38="","",X38*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -2909,11 +2909,11 @@
         <v/>
       </c>
       <c r="X39">
-        <f>IF(OR($E$13&lt;&gt;"OK",M39=""),"",IF(M39&lt;=$A$19,$B$19,IF(M39&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M39-INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M39=""),"",IF(M39&lt;=$A$19,$D$19,IF(M39&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M39-INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M39,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y39">
-        <f>IF(M39="","",$B$5*TAN(RADIANS(M39))*(1+X39/100)*1000/$B$4)</f>
+        <f>IF(X39="","",X39*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3001,11 +3001,11 @@
         <v/>
       </c>
       <c r="X40">
-        <f>IF(OR($E$13&lt;&gt;"OK",M40=""),"",IF(M40&lt;=$A$19,$B$19,IF(M40&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M40-INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M40=""),"",IF(M40&lt;=$A$19,$D$19,IF(M40&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M40-INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M40,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y40">
-        <f>IF(M40="","",$B$5*TAN(RADIANS(M40))*(1+X40/100)*1000/$B$4)</f>
+        <f>IF(X40="","",X40*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3093,11 +3093,11 @@
         <v/>
       </c>
       <c r="X41">
-        <f>IF(OR($E$13&lt;&gt;"OK",M41=""),"",IF(M41&lt;=$A$19,$B$19,IF(M41&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M41-INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M41=""),"",IF(M41&lt;=$A$19,$D$19,IF(M41&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M41-INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M41,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y41">
-        <f>IF(M41="","",$B$5*TAN(RADIANS(M41))*(1+X41/100)*1000/$B$4)</f>
+        <f>IF(X41="","",X41*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3185,11 +3185,11 @@
         <v/>
       </c>
       <c r="X42">
-        <f>IF(OR($E$13&lt;&gt;"OK",M42=""),"",IF(M42&lt;=$A$19,$B$19,IF(M42&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M42-INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M42=""),"",IF(M42&lt;=$A$19,$D$19,IF(M42&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M42-INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M42,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y42">
-        <f>IF(M42="","",$B$5*TAN(RADIANS(M42))*(1+X42/100)*1000/$B$4)</f>
+        <f>IF(X42="","",X42*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3277,11 +3277,11 @@
         <v/>
       </c>
       <c r="X43">
-        <f>IF(OR($E$13&lt;&gt;"OK",M43=""),"",IF(M43&lt;=$A$19,$B$19,IF(M43&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M43-INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M43=""),"",IF(M43&lt;=$A$19,$D$19,IF(M43&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M43-INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M43,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y43">
-        <f>IF(M43="","",$B$5*TAN(RADIANS(M43))*(1+X43/100)*1000/$B$4)</f>
+        <f>IF(X43="","",X43*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3369,11 +3369,11 @@
         <v/>
       </c>
       <c r="X44">
-        <f>IF(OR($E$13&lt;&gt;"OK",M44=""),"",IF(M44&lt;=$A$19,$B$19,IF(M44&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M44-INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M44=""),"",IF(M44&lt;=$A$19,$D$19,IF(M44&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M44-INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M44,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y44">
-        <f>IF(M44="","",$B$5*TAN(RADIANS(M44))*(1+X44/100)*1000/$B$4)</f>
+        <f>IF(X44="","",X44*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3461,11 +3461,11 @@
         <v/>
       </c>
       <c r="X45">
-        <f>IF(OR($E$13&lt;&gt;"OK",M45=""),"",IF(M45&lt;=$A$19,$B$19,IF(M45&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M45-INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M45=""),"",IF(M45&lt;=$A$19,$D$19,IF(M45&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M45-INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M45,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y45">
-        <f>IF(M45="","",$B$5*TAN(RADIANS(M45))*(1+X45/100)*1000/$B$4)</f>
+        <f>IF(X45="","",X45*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3553,11 +3553,11 @@
         <v/>
       </c>
       <c r="X46">
-        <f>IF(OR($E$13&lt;&gt;"OK",M46=""),"",IF(M46&lt;=$A$19,$B$19,IF(M46&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M46-INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M46=""),"",IF(M46&lt;=$A$19,$D$19,IF(M46&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M46-INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M46,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y46">
-        <f>IF(M46="","",$B$5*TAN(RADIANS(M46))*(1+X46/100)*1000/$B$4)</f>
+        <f>IF(X46="","",X46*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3645,11 +3645,11 @@
         <v/>
       </c>
       <c r="X47">
-        <f>IF(OR($E$13&lt;&gt;"OK",M47=""),"",IF(M47&lt;=$A$19,$B$19,IF(M47&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M47-INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M47=""),"",IF(M47&lt;=$A$19,$D$19,IF(M47&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M47-INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M47,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y47">
-        <f>IF(M47="","",$B$5*TAN(RADIANS(M47))*(1+X47/100)*1000/$B$4)</f>
+        <f>IF(X47="","",X47*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3737,11 +3737,11 @@
         <v/>
       </c>
       <c r="X48">
-        <f>IF(OR($E$13&lt;&gt;"OK",M48=""),"",IF(M48&lt;=$A$19,$B$19,IF(M48&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M48-INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M48=""),"",IF(M48&lt;=$A$19,$D$19,IF(M48&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M48-INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M48,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y48">
-        <f>IF(M48="","",$B$5*TAN(RADIANS(M48))*(1+X48/100)*1000/$B$4)</f>
+        <f>IF(X48="","",X48*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3829,11 +3829,11 @@
         <v/>
       </c>
       <c r="X49">
-        <f>IF(OR($E$13&lt;&gt;"OK",M49=""),"",IF(M49&lt;=$A$19,$B$19,IF(M49&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M49-INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M49=""),"",IF(M49&lt;=$A$19,$D$19,IF(M49&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M49-INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M49,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y49">
-        <f>IF(M49="","",$B$5*TAN(RADIANS(M49))*(1+X49/100)*1000/$B$4)</f>
+        <f>IF(X49="","",X49*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -3921,11 +3921,11 @@
         <v/>
       </c>
       <c r="X50">
-        <f>IF(OR($E$13&lt;&gt;"OK",M50=""),"",IF(M50&lt;=$A$19,$B$19,IF(M50&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M50-INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M50=""),"",IF(M50&lt;=$A$19,$D$19,IF(M50&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M50-INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M50,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y50">
-        <f>IF(M50="","",$B$5*TAN(RADIANS(M50))*(1+X50/100)*1000/$B$4)</f>
+        <f>IF(X50="","",X50*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4013,11 +4013,11 @@
         <v/>
       </c>
       <c r="X51">
-        <f>IF(OR($E$13&lt;&gt;"OK",M51=""),"",IF(M51&lt;=$A$19,$B$19,IF(M51&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M51-INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M51=""),"",IF(M51&lt;=$A$19,$D$19,IF(M51&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M51-INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M51,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y51">
-        <f>IF(M51="","",$B$5*TAN(RADIANS(M51))*(1+X51/100)*1000/$B$4)</f>
+        <f>IF(X51="","",X51*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4105,11 +4105,11 @@
         <v/>
       </c>
       <c r="X52">
-        <f>IF(OR($E$13&lt;&gt;"OK",M52=""),"",IF(M52&lt;=$A$19,$B$19,IF(M52&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M52-INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M52=""),"",IF(M52&lt;=$A$19,$D$19,IF(M52&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M52-INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M52,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y52">
-        <f>IF(M52="","",$B$5*TAN(RADIANS(M52))*(1+X52/100)*1000/$B$4)</f>
+        <f>IF(X52="","",X52*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4197,11 +4197,11 @@
         <v/>
       </c>
       <c r="X53">
-        <f>IF(OR($E$13&lt;&gt;"OK",M53=""),"",IF(M53&lt;=$A$19,$B$19,IF(M53&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M53-INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M53=""),"",IF(M53&lt;=$A$19,$D$19,IF(M53&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M53-INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M53,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y53">
-        <f>IF(M53="","",$B$5*TAN(RADIANS(M53))*(1+X53/100)*1000/$B$4)</f>
+        <f>IF(X53="","",X53*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4289,11 +4289,11 @@
         <v/>
       </c>
       <c r="X54">
-        <f>IF(OR($E$13&lt;&gt;"OK",M54=""),"",IF(M54&lt;=$A$19,$B$19,IF(M54&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M54-INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M54=""),"",IF(M54&lt;=$A$19,$D$19,IF(M54&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M54-INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M54,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y54">
-        <f>IF(M54="","",$B$5*TAN(RADIANS(M54))*(1+X54/100)*1000/$B$4)</f>
+        <f>IF(X54="","",X54*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4381,11 +4381,11 @@
         <v/>
       </c>
       <c r="X55">
-        <f>IF(OR($E$13&lt;&gt;"OK",M55=""),"",IF(M55&lt;=$A$19,$B$19,IF(M55&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M55-INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M55=""),"",IF(M55&lt;=$A$19,$D$19,IF(M55&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M55-INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M55,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y55">
-        <f>IF(M55="","",$B$5*TAN(RADIANS(M55))*(1+X55/100)*1000/$B$4)</f>
+        <f>IF(X55="","",X55*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4473,11 +4473,11 @@
         <v/>
       </c>
       <c r="X56">
-        <f>IF(OR($E$13&lt;&gt;"OK",M56=""),"",IF(M56&lt;=$A$19,$B$19,IF(M56&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M56-INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M56=""),"",IF(M56&lt;=$A$19,$D$19,IF(M56&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M56-INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M56,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y56">
-        <f>IF(M56="","",$B$5*TAN(RADIANS(M56))*(1+X56/100)*1000/$B$4)</f>
+        <f>IF(X56="","",X56*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4565,11 +4565,11 @@
         <v/>
       </c>
       <c r="X57">
-        <f>IF(OR($E$13&lt;&gt;"OK",M57=""),"",IF(M57&lt;=$A$19,$B$19,IF(M57&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M57-INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M57=""),"",IF(M57&lt;=$A$19,$D$19,IF(M57&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M57-INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M57,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y57">
-        <f>IF(M57="","",$B$5*TAN(RADIANS(M57))*(1+X57/100)*1000/$B$4)</f>
+        <f>IF(X57="","",X57*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4657,11 +4657,11 @@
         <v/>
       </c>
       <c r="X58">
-        <f>IF(OR($E$13&lt;&gt;"OK",M58=""),"",IF(M58&lt;=$A$19,$B$19,IF(M58&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M58-INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M58=""),"",IF(M58&lt;=$A$19,$D$19,IF(M58&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M58-INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M58,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y58">
-        <f>IF(M58="","",$B$5*TAN(RADIANS(M58))*(1+X58/100)*1000/$B$4)</f>
+        <f>IF(X58="","",X58*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4749,11 +4749,11 @@
         <v/>
       </c>
       <c r="X59">
-        <f>IF(OR($E$13&lt;&gt;"OK",M59=""),"",IF(M59&lt;=$A$19,$B$19,IF(M59&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M59-INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M59=""),"",IF(M59&lt;=$A$19,$D$19,IF(M59&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M59-INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M59,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y59">
-        <f>IF(M59="","",$B$5*TAN(RADIANS(M59))*(1+X59/100)*1000/$B$4)</f>
+        <f>IF(X59="","",X59*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4841,11 +4841,11 @@
         <v/>
       </c>
       <c r="X60">
-        <f>IF(OR($E$13&lt;&gt;"OK",M60=""),"",IF(M60&lt;=$A$19,$B$19,IF(M60&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M60-INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M60=""),"",IF(M60&lt;=$A$19,$D$19,IF(M60&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M60-INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M60,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y60">
-        <f>IF(M60="","",$B$5*TAN(RADIANS(M60))*(1+X60/100)*1000/$B$4)</f>
+        <f>IF(X60="","",X60*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -4933,11 +4933,11 @@
         <v/>
       </c>
       <c r="X61">
-        <f>IF(OR($E$13&lt;&gt;"OK",M61=""),"",IF(M61&lt;=$A$19,$B$19,IF(M61&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M61-INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M61=""),"",IF(M61&lt;=$A$19,$D$19,IF(M61&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M61-INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M61,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y61">
-        <f>IF(M61="","",$B$5*TAN(RADIANS(M61))*(1+X61/100)*1000/$B$4)</f>
+        <f>IF(X61="","",X61*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5025,11 +5025,11 @@
         <v/>
       </c>
       <c r="X62">
-        <f>IF(OR($E$13&lt;&gt;"OK",M62=""),"",IF(M62&lt;=$A$19,$B$19,IF(M62&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M62-INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M62=""),"",IF(M62&lt;=$A$19,$D$19,IF(M62&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M62-INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M62,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y62">
-        <f>IF(M62="","",$B$5*TAN(RADIANS(M62))*(1+X62/100)*1000/$B$4)</f>
+        <f>IF(X62="","",X62*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5117,11 +5117,11 @@
         <v/>
       </c>
       <c r="X63">
-        <f>IF(OR($E$13&lt;&gt;"OK",M63=""),"",IF(M63&lt;=$A$19,$B$19,IF(M63&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M63-INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M63=""),"",IF(M63&lt;=$A$19,$D$19,IF(M63&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M63-INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M63,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y63">
-        <f>IF(M63="","",$B$5*TAN(RADIANS(M63))*(1+X63/100)*1000/$B$4)</f>
+        <f>IF(X63="","",X63*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5209,11 +5209,11 @@
         <v/>
       </c>
       <c r="X64">
-        <f>IF(OR($E$13&lt;&gt;"OK",M64=""),"",IF(M64&lt;=$A$19,$B$19,IF(M64&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M64-INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M64=""),"",IF(M64&lt;=$A$19,$D$19,IF(M64&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M64-INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M64,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y64">
-        <f>IF(M64="","",$B$5*TAN(RADIANS(M64))*(1+X64/100)*1000/$B$4)</f>
+        <f>IF(X64="","",X64*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5301,11 +5301,11 @@
         <v/>
       </c>
       <c r="X65">
-        <f>IF(OR($E$13&lt;&gt;"OK",M65=""),"",IF(M65&lt;=$A$19,$B$19,IF(M65&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M65-INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M65=""),"",IF(M65&lt;=$A$19,$D$19,IF(M65&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M65-INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M65,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y65">
-        <f>IF(M65="","",$B$5*TAN(RADIANS(M65))*(1+X65/100)*1000/$B$4)</f>
+        <f>IF(X65="","",X65*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5393,11 +5393,11 @@
         <v/>
       </c>
       <c r="X66">
-        <f>IF(OR($E$13&lt;&gt;"OK",M66=""),"",IF(M66&lt;=$A$19,$B$19,IF(M66&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M66-INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M66=""),"",IF(M66&lt;=$A$19,$D$19,IF(M66&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M66-INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M66,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y66">
-        <f>IF(M66="","",$B$5*TAN(RADIANS(M66))*(1+X66/100)*1000/$B$4)</f>
+        <f>IF(X66="","",X66*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5485,11 +5485,11 @@
         <v/>
       </c>
       <c r="X67">
-        <f>IF(OR($E$13&lt;&gt;"OK",M67=""),"",IF(M67&lt;=$A$19,$B$19,IF(M67&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M67-INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M67=""),"",IF(M67&lt;=$A$19,$D$19,IF(M67&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M67-INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M67,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y67">
-        <f>IF(M67="","",$B$5*TAN(RADIANS(M67))*(1+X67/100)*1000/$B$4)</f>
+        <f>IF(X67="","",X67*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5577,11 +5577,11 @@
         <v/>
       </c>
       <c r="X68">
-        <f>IF(OR($E$13&lt;&gt;"OK",M68=""),"",IF(M68&lt;=$A$19,$B$19,IF(M68&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M68-INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M68=""),"",IF(M68&lt;=$A$19,$D$19,IF(M68&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M68-INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M68,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y68">
-        <f>IF(M68="","",$B$5*TAN(RADIANS(M68))*(1+X68/100)*1000/$B$4)</f>
+        <f>IF(X68="","",X68*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5669,11 +5669,11 @@
         <v/>
       </c>
       <c r="X69">
-        <f>IF(OR($E$13&lt;&gt;"OK",M69=""),"",IF(M69&lt;=$A$19,$B$19,IF(M69&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M69-INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M69=""),"",IF(M69&lt;=$A$19,$D$19,IF(M69&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M69-INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M69,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y69">
-        <f>IF(M69="","",$B$5*TAN(RADIANS(M69))*(1+X69/100)*1000/$B$4)</f>
+        <f>IF(X69="","",X69*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5761,11 +5761,11 @@
         <v/>
       </c>
       <c r="X70">
-        <f>IF(OR($E$13&lt;&gt;"OK",M70=""),"",IF(M70&lt;=$A$19,$B$19,IF(M70&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M70-INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M70=""),"",IF(M70&lt;=$A$19,$D$19,IF(M70&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M70-INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M70,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y70">
-        <f>IF(M70="","",$B$5*TAN(RADIANS(M70))*(1+X70/100)*1000/$B$4)</f>
+        <f>IF(X70="","",X70*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5853,11 +5853,11 @@
         <v/>
       </c>
       <c r="X71">
-        <f>IF(OR($E$13&lt;&gt;"OK",M71=""),"",IF(M71&lt;=$A$19,$B$19,IF(M71&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M71-INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M71=""),"",IF(M71&lt;=$A$19,$D$19,IF(M71&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M71-INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M71,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y71">
-        <f>IF(M71="","",$B$5*TAN(RADIANS(M71))*(1+X71/100)*1000/$B$4)</f>
+        <f>IF(X71="","",X71*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -5945,11 +5945,11 @@
         <v/>
       </c>
       <c r="X72">
-        <f>IF(OR($E$13&lt;&gt;"OK",M72=""),"",IF(M72&lt;=$A$19,$B$19,IF(M72&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M72-INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M72=""),"",IF(M72&lt;=$A$19,$D$19,IF(M72&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M72-INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M72,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y72">
-        <f>IF(M72="","",$B$5*TAN(RADIANS(M72))*(1+X72/100)*1000/$B$4)</f>
+        <f>IF(X72="","",X72*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6037,11 +6037,11 @@
         <v/>
       </c>
       <c r="X73">
-        <f>IF(OR($E$13&lt;&gt;"OK",M73=""),"",IF(M73&lt;=$A$19,$B$19,IF(M73&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M73-INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M73=""),"",IF(M73&lt;=$A$19,$D$19,IF(M73&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M73-INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M73,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y73">
-        <f>IF(M73="","",$B$5*TAN(RADIANS(M73))*(1+X73/100)*1000/$B$4)</f>
+        <f>IF(X73="","",X73*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6129,11 +6129,11 @@
         <v/>
       </c>
       <c r="X74">
-        <f>IF(OR($E$13&lt;&gt;"OK",M74=""),"",IF(M74&lt;=$A$19,$B$19,IF(M74&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M74-INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M74=""),"",IF(M74&lt;=$A$19,$D$19,IF(M74&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M74-INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M74,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y74">
-        <f>IF(M74="","",$B$5*TAN(RADIANS(M74))*(1+X74/100)*1000/$B$4)</f>
+        <f>IF(X74="","",X74*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6221,11 +6221,11 @@
         <v/>
       </c>
       <c r="X75">
-        <f>IF(OR($E$13&lt;&gt;"OK",M75=""),"",IF(M75&lt;=$A$19,$B$19,IF(M75&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M75-INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M75=""),"",IF(M75&lt;=$A$19,$D$19,IF(M75&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M75-INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M75,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y75">
-        <f>IF(M75="","",$B$5*TAN(RADIANS(M75))*(1+X75/100)*1000/$B$4)</f>
+        <f>IF(X75="","",X75*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6313,11 +6313,11 @@
         <v/>
       </c>
       <c r="X76">
-        <f>IF(OR($E$13&lt;&gt;"OK",M76=""),"",IF(M76&lt;=$A$19,$B$19,IF(M76&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M76-INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M76=""),"",IF(M76&lt;=$A$19,$D$19,IF(M76&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M76-INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M76,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y76">
-        <f>IF(M76="","",$B$5*TAN(RADIANS(M76))*(1+X76/100)*1000/$B$4)</f>
+        <f>IF(X76="","",X76*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6405,11 +6405,11 @@
         <v/>
       </c>
       <c r="X77">
-        <f>IF(OR($E$13&lt;&gt;"OK",M77=""),"",IF(M77&lt;=$A$19,$B$19,IF(M77&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M77-INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M77=""),"",IF(M77&lt;=$A$19,$D$19,IF(M77&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M77-INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M77,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y77">
-        <f>IF(M77="","",$B$5*TAN(RADIANS(M77))*(1+X77/100)*1000/$B$4)</f>
+        <f>IF(X77="","",X77*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6497,11 +6497,11 @@
         <v/>
       </c>
       <c r="X78">
-        <f>IF(OR($E$13&lt;&gt;"OK",M78=""),"",IF(M78&lt;=$A$19,$B$19,IF(M78&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M78-INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M78=""),"",IF(M78&lt;=$A$19,$D$19,IF(M78&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M78-INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M78,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y78">
-        <f>IF(M78="","",$B$5*TAN(RADIANS(M78))*(1+X78/100)*1000/$B$4)</f>
+        <f>IF(X78="","",X78*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6589,11 +6589,11 @@
         <v/>
       </c>
       <c r="X79">
-        <f>IF(OR($E$13&lt;&gt;"OK",M79=""),"",IF(M79&lt;=$A$19,$B$19,IF(M79&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M79-INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M79=""),"",IF(M79&lt;=$A$19,$D$19,IF(M79&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M79-INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M79,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y79">
-        <f>IF(M79="","",$B$5*TAN(RADIANS(M79))*(1+X79/100)*1000/$B$4)</f>
+        <f>IF(X79="","",X79*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6681,11 +6681,11 @@
         <v/>
       </c>
       <c r="X80">
-        <f>IF(OR($E$13&lt;&gt;"OK",M80=""),"",IF(M80&lt;=$A$19,$B$19,IF(M80&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M80-INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M80=""),"",IF(M80&lt;=$A$19,$D$19,IF(M80&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M80-INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M80,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y80">
-        <f>IF(M80="","",$B$5*TAN(RADIANS(M80))*(1+X80/100)*1000/$B$4)</f>
+        <f>IF(X80="","",X80*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6773,11 +6773,11 @@
         <v/>
       </c>
       <c r="X81">
-        <f>IF(OR($E$13&lt;&gt;"OK",M81=""),"",IF(M81&lt;=$A$19,$B$19,IF(M81&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M81-INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M81=""),"",IF(M81&lt;=$A$19,$D$19,IF(M81&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M81-INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M81,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y81">
-        <f>IF(M81="","",$B$5*TAN(RADIANS(M81))*(1+X81/100)*1000/$B$4)</f>
+        <f>IF(X81="","",X81*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6865,11 +6865,11 @@
         <v/>
       </c>
       <c r="X82">
-        <f>IF(OR($E$13&lt;&gt;"OK",M82=""),"",IF(M82&lt;=$A$19,$B$19,IF(M82&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M82-INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M82=""),"",IF(M82&lt;=$A$19,$D$19,IF(M82&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M82-INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M82,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y82">
-        <f>IF(M82="","",$B$5*TAN(RADIANS(M82))*(1+X82/100)*1000/$B$4)</f>
+        <f>IF(X82="","",X82*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -6957,11 +6957,11 @@
         <v/>
       </c>
       <c r="X83">
-        <f>IF(OR($E$13&lt;&gt;"OK",M83=""),"",IF(M83&lt;=$A$19,$B$19,IF(M83&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M83-INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M83=""),"",IF(M83&lt;=$A$19,$D$19,IF(M83&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M83-INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M83,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y83">
-        <f>IF(M83="","",$B$5*TAN(RADIANS(M83))*(1+X83/100)*1000/$B$4)</f>
+        <f>IF(X83="","",X83*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7049,11 +7049,11 @@
         <v/>
       </c>
       <c r="X84">
-        <f>IF(OR($E$13&lt;&gt;"OK",M84=""),"",IF(M84&lt;=$A$19,$B$19,IF(M84&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M84-INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M84=""),"",IF(M84&lt;=$A$19,$D$19,IF(M84&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M84-INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M84,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y84">
-        <f>IF(M84="","",$B$5*TAN(RADIANS(M84))*(1+X84/100)*1000/$B$4)</f>
+        <f>IF(X84="","",X84*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7141,11 +7141,11 @@
         <v/>
       </c>
       <c r="X85">
-        <f>IF(OR($E$13&lt;&gt;"OK",M85=""),"",IF(M85&lt;=$A$19,$B$19,IF(M85&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M85-INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M85=""),"",IF(M85&lt;=$A$19,$D$19,IF(M85&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M85-INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M85,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y85">
-        <f>IF(M85="","",$B$5*TAN(RADIANS(M85))*(1+X85/100)*1000/$B$4)</f>
+        <f>IF(X85="","",X85*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7233,11 +7233,11 @@
         <v/>
       </c>
       <c r="X86">
-        <f>IF(OR($E$13&lt;&gt;"OK",M86=""),"",IF(M86&lt;=$A$19,$B$19,IF(M86&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M86-INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M86=""),"",IF(M86&lt;=$A$19,$D$19,IF(M86&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M86-INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M86,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y86">
-        <f>IF(M86="","",$B$5*TAN(RADIANS(M86))*(1+X86/100)*1000/$B$4)</f>
+        <f>IF(X86="","",X86*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7325,11 +7325,11 @@
         <v/>
       </c>
       <c r="X87">
-        <f>IF(OR($E$13&lt;&gt;"OK",M87=""),"",IF(M87&lt;=$A$19,$B$19,IF(M87&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M87-INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M87=""),"",IF(M87&lt;=$A$19,$D$19,IF(M87&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M87-INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M87,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y87">
-        <f>IF(M87="","",$B$5*TAN(RADIANS(M87))*(1+X87/100)*1000/$B$4)</f>
+        <f>IF(X87="","",X87*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7417,11 +7417,11 @@
         <v/>
       </c>
       <c r="X88">
-        <f>IF(OR($E$13&lt;&gt;"OK",M88=""),"",IF(M88&lt;=$A$19,$B$19,IF(M88&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M88-INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M88=""),"",IF(M88&lt;=$A$19,$D$19,IF(M88&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M88-INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M88,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y88">
-        <f>IF(M88="","",$B$5*TAN(RADIANS(M88))*(1+X88/100)*1000/$B$4)</f>
+        <f>IF(X88="","",X88*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7509,11 +7509,11 @@
         <v/>
       </c>
       <c r="X89">
-        <f>IF(OR($E$13&lt;&gt;"OK",M89=""),"",IF(M89&lt;=$A$19,$B$19,IF(M89&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M89-INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M89=""),"",IF(M89&lt;=$A$19,$D$19,IF(M89&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M89-INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M89,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y89">
-        <f>IF(M89="","",$B$5*TAN(RADIANS(M89))*(1+X89/100)*1000/$B$4)</f>
+        <f>IF(X89="","",X89*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7601,11 +7601,11 @@
         <v/>
       </c>
       <c r="X90">
-        <f>IF(OR($E$13&lt;&gt;"OK",M90=""),"",IF(M90&lt;=$A$19,$B$19,IF(M90&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M90-INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M90=""),"",IF(M90&lt;=$A$19,$D$19,IF(M90&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M90-INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M90,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y90">
-        <f>IF(M90="","",$B$5*TAN(RADIANS(M90))*(1+X90/100)*1000/$B$4)</f>
+        <f>IF(X90="","",X90*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7693,11 +7693,11 @@
         <v/>
       </c>
       <c r="X91">
-        <f>IF(OR($E$13&lt;&gt;"OK",M91=""),"",IF(M91&lt;=$A$19,$B$19,IF(M91&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M91-INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M91=""),"",IF(M91&lt;=$A$19,$D$19,IF(M91&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M91-INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M91,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y91">
-        <f>IF(M91="","",$B$5*TAN(RADIANS(M91))*(1+X91/100)*1000/$B$4)</f>
+        <f>IF(X91="","",X91*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7785,11 +7785,11 @@
         <v/>
       </c>
       <c r="X92">
-        <f>IF(OR($E$13&lt;&gt;"OK",M92=""),"",IF(M92&lt;=$A$19,$B$19,IF(M92&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M92-INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M92=""),"",IF(M92&lt;=$A$19,$D$19,IF(M92&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M92-INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M92,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y92">
-        <f>IF(M92="","",$B$5*TAN(RADIANS(M92))*(1+X92/100)*1000/$B$4)</f>
+        <f>IF(X92="","",X92*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7877,11 +7877,11 @@
         <v/>
       </c>
       <c r="X93">
-        <f>IF(OR($E$13&lt;&gt;"OK",M93=""),"",IF(M93&lt;=$A$19,$B$19,IF(M93&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M93-INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M93=""),"",IF(M93&lt;=$A$19,$D$19,IF(M93&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M93-INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M93,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y93">
-        <f>IF(M93="","",$B$5*TAN(RADIANS(M93))*(1+X93/100)*1000/$B$4)</f>
+        <f>IF(X93="","",X93*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -7969,11 +7969,11 @@
         <v/>
       </c>
       <c r="X94">
-        <f>IF(OR($E$13&lt;&gt;"OK",M94=""),"",IF(M94&lt;=$A$19,$B$19,IF(M94&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M94-INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M94=""),"",IF(M94&lt;=$A$19,$D$19,IF(M94&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M94-INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M94,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y94">
-        <f>IF(M94="","",$B$5*TAN(RADIANS(M94))*(1+X94/100)*1000/$B$4)</f>
+        <f>IF(X94="","",X94*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8061,11 +8061,11 @@
         <v/>
       </c>
       <c r="X95">
-        <f>IF(OR($E$13&lt;&gt;"OK",M95=""),"",IF(M95&lt;=$A$19,$B$19,IF(M95&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M95-INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M95=""),"",IF(M95&lt;=$A$19,$D$19,IF(M95&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M95-INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M95,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y95">
-        <f>IF(M95="","",$B$5*TAN(RADIANS(M95))*(1+X95/100)*1000/$B$4)</f>
+        <f>IF(X95="","",X95*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8153,11 +8153,11 @@
         <v/>
       </c>
       <c r="X96">
-        <f>IF(OR($E$13&lt;&gt;"OK",M96=""),"",IF(M96&lt;=$A$19,$B$19,IF(M96&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M96-INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M96=""),"",IF(M96&lt;=$A$19,$D$19,IF(M96&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M96-INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M96,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y96">
-        <f>IF(M96="","",$B$5*TAN(RADIANS(M96))*(1+X96/100)*1000/$B$4)</f>
+        <f>IF(X96="","",X96*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8245,11 +8245,11 @@
         <v/>
       </c>
       <c r="X97">
-        <f>IF(OR($E$13&lt;&gt;"OK",M97=""),"",IF(M97&lt;=$A$19,$B$19,IF(M97&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M97-INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M97=""),"",IF(M97&lt;=$A$19,$D$19,IF(M97&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M97-INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M97,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y97">
-        <f>IF(M97="","",$B$5*TAN(RADIANS(M97))*(1+X97/100)*1000/$B$4)</f>
+        <f>IF(X97="","",X97*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8337,11 +8337,11 @@
         <v/>
       </c>
       <c r="X98">
-        <f>IF(OR($E$13&lt;&gt;"OK",M98=""),"",IF(M98&lt;=$A$19,$B$19,IF(M98&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M98-INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M98=""),"",IF(M98&lt;=$A$19,$D$19,IF(M98&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M98-INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M98,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y98">
-        <f>IF(M98="","",$B$5*TAN(RADIANS(M98))*(1+X98/100)*1000/$B$4)</f>
+        <f>IF(X98="","",X98*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8429,11 +8429,11 @@
         <v/>
       </c>
       <c r="X99">
-        <f>IF(OR($E$13&lt;&gt;"OK",M99=""),"",IF(M99&lt;=$A$19,$B$19,IF(M99&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M99-INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M99=""),"",IF(M99&lt;=$A$19,$D$19,IF(M99&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M99-INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M99,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y99">
-        <f>IF(M99="","",$B$5*TAN(RADIANS(M99))*(1+X99/100)*1000/$B$4)</f>
+        <f>IF(X99="","",X99*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8521,11 +8521,11 @@
         <v/>
       </c>
       <c r="X100">
-        <f>IF(OR($E$13&lt;&gt;"OK",M100=""),"",IF(M100&lt;=$A$19,$B$19,IF(M100&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M100-INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M100=""),"",IF(M100&lt;=$A$19,$D$19,IF(M100&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M100-INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M100,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y100">
-        <f>IF(M100="","",$B$5*TAN(RADIANS(M100))*(1+X100/100)*1000/$B$4)</f>
+        <f>IF(X100="","",X100*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8613,11 +8613,11 @@
         <v/>
       </c>
       <c r="X101">
-        <f>IF(OR($E$13&lt;&gt;"OK",M101=""),"",IF(M101&lt;=$A$19,$B$19,IF(M101&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M101-INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M101=""),"",IF(M101&lt;=$A$19,$D$19,IF(M101&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M101-INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M101,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y101">
-        <f>IF(M101="","",$B$5*TAN(RADIANS(M101))*(1+X101/100)*1000/$B$4)</f>
+        <f>IF(X101="","",X101*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8705,11 +8705,11 @@
         <v/>
       </c>
       <c r="X102">
-        <f>IF(OR($E$13&lt;&gt;"OK",M102=""),"",IF(M102&lt;=$A$19,$B$19,IF(M102&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M102-INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M102=""),"",IF(M102&lt;=$A$19,$D$19,IF(M102&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M102-INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M102,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y102">
-        <f>IF(M102="","",$B$5*TAN(RADIANS(M102))*(1+X102/100)*1000/$B$4)</f>
+        <f>IF(X102="","",X102*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8797,11 +8797,11 @@
         <v/>
       </c>
       <c r="X103">
-        <f>IF(OR($E$13&lt;&gt;"OK",M103=""),"",IF(M103&lt;=$A$19,$B$19,IF(M103&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M103-INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M103=""),"",IF(M103&lt;=$A$19,$D$19,IF(M103&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M103-INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M103,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y103">
-        <f>IF(M103="","",$B$5*TAN(RADIANS(M103))*(1+X103/100)*1000/$B$4)</f>
+        <f>IF(X103="","",X103*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8889,11 +8889,11 @@
         <v/>
       </c>
       <c r="X104">
-        <f>IF(OR($E$13&lt;&gt;"OK",M104=""),"",IF(M104&lt;=$A$19,$B$19,IF(M104&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M104-INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M104=""),"",IF(M104&lt;=$A$19,$D$19,IF(M104&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M104-INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M104,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y104">
-        <f>IF(M104="","",$B$5*TAN(RADIANS(M104))*(1+X104/100)*1000/$B$4)</f>
+        <f>IF(X104="","",X104*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -8981,11 +8981,11 @@
         <v/>
       </c>
       <c r="X105">
-        <f>IF(OR($E$13&lt;&gt;"OK",M105=""),"",IF(M105&lt;=$A$19,$B$19,IF(M105&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M105-INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M105=""),"",IF(M105&lt;=$A$19,$D$19,IF(M105&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M105-INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M105,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y105">
-        <f>IF(M105="","",$B$5*TAN(RADIANS(M105))*(1+X105/100)*1000/$B$4)</f>
+        <f>IF(X105="","",X105*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9073,11 +9073,11 @@
         <v/>
       </c>
       <c r="X106">
-        <f>IF(OR($E$13&lt;&gt;"OK",M106=""),"",IF(M106&lt;=$A$19,$B$19,IF(M106&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M106-INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M106=""),"",IF(M106&lt;=$A$19,$D$19,IF(M106&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M106-INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M106,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y106">
-        <f>IF(M106="","",$B$5*TAN(RADIANS(M106))*(1+X106/100)*1000/$B$4)</f>
+        <f>IF(X106="","",X106*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9165,11 +9165,11 @@
         <v/>
       </c>
       <c r="X107">
-        <f>IF(OR($E$13&lt;&gt;"OK",M107=""),"",IF(M107&lt;=$A$19,$B$19,IF(M107&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M107-INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M107=""),"",IF(M107&lt;=$A$19,$D$19,IF(M107&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M107-INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M107,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y107">
-        <f>IF(M107="","",$B$5*TAN(RADIANS(M107))*(1+X107/100)*1000/$B$4)</f>
+        <f>IF(X107="","",X107*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9257,11 +9257,11 @@
         <v/>
       </c>
       <c r="X108">
-        <f>IF(OR($E$13&lt;&gt;"OK",M108=""),"",IF(M108&lt;=$A$19,$B$19,IF(M108&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M108-INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M108=""),"",IF(M108&lt;=$A$19,$D$19,IF(M108&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M108-INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M108,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y108">
-        <f>IF(M108="","",$B$5*TAN(RADIANS(M108))*(1+X108/100)*1000/$B$4)</f>
+        <f>IF(X108="","",X108*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9349,11 +9349,11 @@
         <v/>
       </c>
       <c r="X109">
-        <f>IF(OR($E$13&lt;&gt;"OK",M109=""),"",IF(M109&lt;=$A$19,$B$19,IF(M109&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M109-INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M109=""),"",IF(M109&lt;=$A$19,$D$19,IF(M109&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M109-INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M109,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y109">
-        <f>IF(M109="","",$B$5*TAN(RADIANS(M109))*(1+X109/100)*1000/$B$4)</f>
+        <f>IF(X109="","",X109*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9441,11 +9441,11 @@
         <v/>
       </c>
       <c r="X110">
-        <f>IF(OR($E$13&lt;&gt;"OK",M110=""),"",IF(M110&lt;=$A$19,$B$19,IF(M110&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M110-INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M110=""),"",IF(M110&lt;=$A$19,$D$19,IF(M110&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M110-INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M110,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y110">
-        <f>IF(M110="","",$B$5*TAN(RADIANS(M110))*(1+X110/100)*1000/$B$4)</f>
+        <f>IF(X110="","",X110*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9533,11 +9533,11 @@
         <v/>
       </c>
       <c r="X111">
-        <f>IF(OR($E$13&lt;&gt;"OK",M111=""),"",IF(M111&lt;=$A$19,$B$19,IF(M111&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M111-INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M111=""),"",IF(M111&lt;=$A$19,$D$19,IF(M111&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M111-INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M111,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y111">
-        <f>IF(M111="","",$B$5*TAN(RADIANS(M111))*(1+X111/100)*1000/$B$4)</f>
+        <f>IF(X111="","",X111*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9625,11 +9625,11 @@
         <v/>
       </c>
       <c r="X112">
-        <f>IF(OR($E$13&lt;&gt;"OK",M112=""),"",IF(M112&lt;=$A$19,$B$19,IF(M112&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M112-INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M112=""),"",IF(M112&lt;=$A$19,$D$19,IF(M112&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M112-INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M112,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y112">
-        <f>IF(M112="","",$B$5*TAN(RADIANS(M112))*(1+X112/100)*1000/$B$4)</f>
+        <f>IF(X112="","",X112*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9717,11 +9717,11 @@
         <v/>
       </c>
       <c r="X113">
-        <f>IF(OR($E$13&lt;&gt;"OK",M113=""),"",IF(M113&lt;=$A$19,$B$19,IF(M113&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M113-INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M113=""),"",IF(M113&lt;=$A$19,$D$19,IF(M113&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M113-INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M113,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y113">
-        <f>IF(M113="","",$B$5*TAN(RADIANS(M113))*(1+X113/100)*1000/$B$4)</f>
+        <f>IF(X113="","",X113*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9809,11 +9809,11 @@
         <v/>
       </c>
       <c r="X114">
-        <f>IF(OR($E$13&lt;&gt;"OK",M114=""),"",IF(M114&lt;=$A$19,$B$19,IF(M114&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M114-INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M114=""),"",IF(M114&lt;=$A$19,$D$19,IF(M114&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M114-INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M114,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y114">
-        <f>IF(M114="","",$B$5*TAN(RADIANS(M114))*(1+X114/100)*1000/$B$4)</f>
+        <f>IF(X114="","",X114*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9901,11 +9901,11 @@
         <v/>
       </c>
       <c r="X115">
-        <f>IF(OR($E$13&lt;&gt;"OK",M115=""),"",IF(M115&lt;=$A$19,$B$19,IF(M115&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M115-INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M115=""),"",IF(M115&lt;=$A$19,$D$19,IF(M115&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M115-INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M115,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y115">
-        <f>IF(M115="","",$B$5*TAN(RADIANS(M115))*(1+X115/100)*1000/$B$4)</f>
+        <f>IF(X115="","",X115*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -9993,11 +9993,11 @@
         <v/>
       </c>
       <c r="X116">
-        <f>IF(OR($E$13&lt;&gt;"OK",M116=""),"",IF(M116&lt;=$A$19,$B$19,IF(M116&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M116-INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M116=""),"",IF(M116&lt;=$A$19,$D$19,IF(M116&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M116-INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M116,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y116">
-        <f>IF(M116="","",$B$5*TAN(RADIANS(M116))*(1+X116/100)*1000/$B$4)</f>
+        <f>IF(X116="","",X116*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10085,11 +10085,11 @@
         <v/>
       </c>
       <c r="X117">
-        <f>IF(OR($E$13&lt;&gt;"OK",M117=""),"",IF(M117&lt;=$A$19,$B$19,IF(M117&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M117-INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M117=""),"",IF(M117&lt;=$A$19,$D$19,IF(M117&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M117-INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M117,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y117">
-        <f>IF(M117="","",$B$5*TAN(RADIANS(M117))*(1+X117/100)*1000/$B$4)</f>
+        <f>IF(X117="","",X117*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10177,11 +10177,11 @@
         <v/>
       </c>
       <c r="X118">
-        <f>IF(OR($E$13&lt;&gt;"OK",M118=""),"",IF(M118&lt;=$A$19,$B$19,IF(M118&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M118-INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M118=""),"",IF(M118&lt;=$A$19,$D$19,IF(M118&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M118-INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M118,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y118">
-        <f>IF(M118="","",$B$5*TAN(RADIANS(M118))*(1+X118/100)*1000/$B$4)</f>
+        <f>IF(X118="","",X118*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10269,11 +10269,11 @@
         <v/>
       </c>
       <c r="X119">
-        <f>IF(OR($E$13&lt;&gt;"OK",M119=""),"",IF(M119&lt;=$A$19,$B$19,IF(M119&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M119-INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M119=""),"",IF(M119&lt;=$A$19,$D$19,IF(M119&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M119-INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M119,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y119">
-        <f>IF(M119="","",$B$5*TAN(RADIANS(M119))*(1+X119/100)*1000/$B$4)</f>
+        <f>IF(X119="","",X119*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10361,11 +10361,11 @@
         <v/>
       </c>
       <c r="X120">
-        <f>IF(OR($E$13&lt;&gt;"OK",M120=""),"",IF(M120&lt;=$A$19,$B$19,IF(M120&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M120-INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M120=""),"",IF(M120&lt;=$A$19,$D$19,IF(M120&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M120-INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M120,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y120">
-        <f>IF(M120="","",$B$5*TAN(RADIANS(M120))*(1+X120/100)*1000/$B$4)</f>
+        <f>IF(X120="","",X120*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10453,11 +10453,11 @@
         <v/>
       </c>
       <c r="X121">
-        <f>IF(OR($E$13&lt;&gt;"OK",M121=""),"",IF(M121&lt;=$A$19,$B$19,IF(M121&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M121-INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M121=""),"",IF(M121&lt;=$A$19,$D$19,IF(M121&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M121-INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M121,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y121">
-        <f>IF(M121="","",$B$5*TAN(RADIANS(M121))*(1+X121/100)*1000/$B$4)</f>
+        <f>IF(X121="","",X121*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10545,11 +10545,11 @@
         <v/>
       </c>
       <c r="X122">
-        <f>IF(OR($E$13&lt;&gt;"OK",M122=""),"",IF(M122&lt;=$A$19,$B$19,IF(M122&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M122-INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M122=""),"",IF(M122&lt;=$A$19,$D$19,IF(M122&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M122-INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M122,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y122">
-        <f>IF(M122="","",$B$5*TAN(RADIANS(M122))*(1+X122/100)*1000/$B$4)</f>
+        <f>IF(X122="","",X122*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10637,11 +10637,11 @@
         <v/>
       </c>
       <c r="X123">
-        <f>IF(OR($E$13&lt;&gt;"OK",M123=""),"",IF(M123&lt;=$A$19,$B$19,IF(M123&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M123-INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M123=""),"",IF(M123&lt;=$A$19,$D$19,IF(M123&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M123-INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M123,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y123">
-        <f>IF(M123="","",$B$5*TAN(RADIANS(M123))*(1+X123/100)*1000/$B$4)</f>
+        <f>IF(X123="","",X123*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10729,11 +10729,11 @@
         <v/>
       </c>
       <c r="X124">
-        <f>IF(OR($E$13&lt;&gt;"OK",M124=""),"",IF(M124&lt;=$A$19,$B$19,IF(M124&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M124-INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M124=""),"",IF(M124&lt;=$A$19,$D$19,IF(M124&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M124-INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M124,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y124">
-        <f>IF(M124="","",$B$5*TAN(RADIANS(M124))*(1+X124/100)*1000/$B$4)</f>
+        <f>IF(X124="","",X124*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10821,11 +10821,11 @@
         <v/>
       </c>
       <c r="X125">
-        <f>IF(OR($E$13&lt;&gt;"OK",M125=""),"",IF(M125&lt;=$A$19,$B$19,IF(M125&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M125-INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M125=""),"",IF(M125&lt;=$A$19,$D$19,IF(M125&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M125-INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M125,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y125">
-        <f>IF(M125="","",$B$5*TAN(RADIANS(M125))*(1+X125/100)*1000/$B$4)</f>
+        <f>IF(X125="","",X125*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -10913,11 +10913,11 @@
         <v/>
       </c>
       <c r="X126">
-        <f>IF(OR($E$13&lt;&gt;"OK",M126=""),"",IF(M126&lt;=$A$19,$B$19,IF(M126&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M126-INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M126=""),"",IF(M126&lt;=$A$19,$D$19,IF(M126&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M126-INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M126,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y126">
-        <f>IF(M126="","",$B$5*TAN(RADIANS(M126))*(1+X126/100)*1000/$B$4)</f>
+        <f>IF(X126="","",X126*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11005,11 +11005,11 @@
         <v/>
       </c>
       <c r="X127">
-        <f>IF(OR($E$13&lt;&gt;"OK",M127=""),"",IF(M127&lt;=$A$19,$B$19,IF(M127&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M127-INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M127=""),"",IF(M127&lt;=$A$19,$D$19,IF(M127&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M127-INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M127,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y127">
-        <f>IF(M127="","",$B$5*TAN(RADIANS(M127))*(1+X127/100)*1000/$B$4)</f>
+        <f>IF(X127="","",X127*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11097,11 +11097,11 @@
         <v/>
       </c>
       <c r="X128">
-        <f>IF(OR($E$13&lt;&gt;"OK",M128=""),"",IF(M128&lt;=$A$19,$B$19,IF(M128&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M128-INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M128=""),"",IF(M128&lt;=$A$19,$D$19,IF(M128&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M128-INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M128,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y128">
-        <f>IF(M128="","",$B$5*TAN(RADIANS(M128))*(1+X128/100)*1000/$B$4)</f>
+        <f>IF(X128="","",X128*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11189,11 +11189,11 @@
         <v/>
       </c>
       <c r="X129">
-        <f>IF(OR($E$13&lt;&gt;"OK",M129=""),"",IF(M129&lt;=$A$19,$B$19,IF(M129&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M129-INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M129=""),"",IF(M129&lt;=$A$19,$D$19,IF(M129&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M129-INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M129,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y129">
-        <f>IF(M129="","",$B$5*TAN(RADIANS(M129))*(1+X129/100)*1000/$B$4)</f>
+        <f>IF(X129="","",X129*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11281,11 +11281,11 @@
         <v/>
       </c>
       <c r="X130">
-        <f>IF(OR($E$13&lt;&gt;"OK",M130=""),"",IF(M130&lt;=$A$19,$B$19,IF(M130&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M130-INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M130=""),"",IF(M130&lt;=$A$19,$D$19,IF(M130&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M130-INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M130,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y130">
-        <f>IF(M130="","",$B$5*TAN(RADIANS(M130))*(1+X130/100)*1000/$B$4)</f>
+        <f>IF(X130="","",X130*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11373,11 +11373,11 @@
         <v/>
       </c>
       <c r="X131">
-        <f>IF(OR($E$13&lt;&gt;"OK",M131=""),"",IF(M131&lt;=$A$19,$B$19,IF(M131&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M131-INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M131=""),"",IF(M131&lt;=$A$19,$D$19,IF(M131&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M131-INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M131,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y131">
-        <f>IF(M131="","",$B$5*TAN(RADIANS(M131))*(1+X131/100)*1000/$B$4)</f>
+        <f>IF(X131="","",X131*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11465,11 +11465,11 @@
         <v/>
       </c>
       <c r="X132">
-        <f>IF(OR($E$13&lt;&gt;"OK",M132=""),"",IF(M132&lt;=$A$19,$B$19,IF(M132&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M132-INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M132=""),"",IF(M132&lt;=$A$19,$D$19,IF(M132&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M132-INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M132,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y132">
-        <f>IF(M132="","",$B$5*TAN(RADIANS(M132))*(1+X132/100)*1000/$B$4)</f>
+        <f>IF(X132="","",X132*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v/>
       </c>
       <c r="X133">
-        <f>IF(OR($E$13&lt;&gt;"OK",M133=""),"",IF(M133&lt;=$A$19,$B$19,IF(M133&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M133-INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M133=""),"",IF(M133&lt;=$A$19,$D$19,IF(M133&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M133-INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M133,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y133">
-        <f>IF(M133="","",$B$5*TAN(RADIANS(M133))*(1+X133/100)*1000/$B$4)</f>
+        <f>IF(X133="","",X133*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11649,11 +11649,11 @@
         <v/>
       </c>
       <c r="X134">
-        <f>IF(OR($E$13&lt;&gt;"OK",M134=""),"",IF(M134&lt;=$A$19,$B$19,IF(M134&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M134-INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M134=""),"",IF(M134&lt;=$A$19,$D$19,IF(M134&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M134-INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M134,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y134">
-        <f>IF(M134="","",$B$5*TAN(RADIANS(M134))*(1+X134/100)*1000/$B$4)</f>
+        <f>IF(X134="","",X134*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11741,11 +11741,11 @@
         <v/>
       </c>
       <c r="X135">
-        <f>IF(OR($E$13&lt;&gt;"OK",M135=""),"",IF(M135&lt;=$A$19,$B$19,IF(M135&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M135-INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M135=""),"",IF(M135&lt;=$A$19,$D$19,IF(M135&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M135-INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M135,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y135">
-        <f>IF(M135="","",$B$5*TAN(RADIANS(M135))*(1+X135/100)*1000/$B$4)</f>
+        <f>IF(X135="","",X135*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11833,11 +11833,11 @@
         <v/>
       </c>
       <c r="X136">
-        <f>IF(OR($E$13&lt;&gt;"OK",M136=""),"",IF(M136&lt;=$A$19,$B$19,IF(M136&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M136-INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M136=""),"",IF(M136&lt;=$A$19,$D$19,IF(M136&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M136-INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M136,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y136">
-        <f>IF(M136="","",$B$5*TAN(RADIANS(M136))*(1+X136/100)*1000/$B$4)</f>
+        <f>IF(X136="","",X136*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -11925,11 +11925,11 @@
         <v/>
       </c>
       <c r="X137">
-        <f>IF(OR($E$13&lt;&gt;"OK",M137=""),"",IF(M137&lt;=$A$19,$B$19,IF(M137&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M137-INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M137=""),"",IF(M137&lt;=$A$19,$D$19,IF(M137&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M137-INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M137,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y137">
-        <f>IF(M137="","",$B$5*TAN(RADIANS(M137))*(1+X137/100)*1000/$B$4)</f>
+        <f>IF(X137="","",X137*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12017,11 +12017,11 @@
         <v/>
       </c>
       <c r="X138">
-        <f>IF(OR($E$13&lt;&gt;"OK",M138=""),"",IF(M138&lt;=$A$19,$B$19,IF(M138&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M138-INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M138=""),"",IF(M138&lt;=$A$19,$D$19,IF(M138&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M138-INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M138,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y138">
-        <f>IF(M138="","",$B$5*TAN(RADIANS(M138))*(1+X138/100)*1000/$B$4)</f>
+        <f>IF(X138="","",X138*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12109,11 +12109,11 @@
         <v/>
       </c>
       <c r="X139">
-        <f>IF(OR($E$13&lt;&gt;"OK",M139=""),"",IF(M139&lt;=$A$19,$B$19,IF(M139&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M139-INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M139=""),"",IF(M139&lt;=$A$19,$D$19,IF(M139&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M139-INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M139,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y139">
-        <f>IF(M139="","",$B$5*TAN(RADIANS(M139))*(1+X139/100)*1000/$B$4)</f>
+        <f>IF(X139="","",X139*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12201,11 +12201,11 @@
         <v/>
       </c>
       <c r="X140">
-        <f>IF(OR($E$13&lt;&gt;"OK",M140=""),"",IF(M140&lt;=$A$19,$B$19,IF(M140&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M140-INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M140=""),"",IF(M140&lt;=$A$19,$D$19,IF(M140&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M140-INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M140,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y140">
-        <f>IF(M140="","",$B$5*TAN(RADIANS(M140))*(1+X140/100)*1000/$B$4)</f>
+        <f>IF(X140="","",X140*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12293,11 +12293,11 @@
         <v/>
       </c>
       <c r="X141">
-        <f>IF(OR($E$13&lt;&gt;"OK",M141=""),"",IF(M141&lt;=$A$19,$B$19,IF(M141&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M141-INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M141=""),"",IF(M141&lt;=$A$19,$D$19,IF(M141&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M141-INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M141,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y141">
-        <f>IF(M141="","",$B$5*TAN(RADIANS(M141))*(1+X141/100)*1000/$B$4)</f>
+        <f>IF(X141="","",X141*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12385,11 +12385,11 @@
         <v/>
       </c>
       <c r="X142">
-        <f>IF(OR($E$13&lt;&gt;"OK",M142=""),"",IF(M142&lt;=$A$19,$B$19,IF(M142&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M142-INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M142=""),"",IF(M142&lt;=$A$19,$D$19,IF(M142&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M142-INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M142,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y142">
-        <f>IF(M142="","",$B$5*TAN(RADIANS(M142))*(1+X142/100)*1000/$B$4)</f>
+        <f>IF(X142="","",X142*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12477,11 +12477,11 @@
         <v/>
       </c>
       <c r="X143">
-        <f>IF(OR($E$13&lt;&gt;"OK",M143=""),"",IF(M143&lt;=$A$19,$B$19,IF(M143&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M143-INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M143=""),"",IF(M143&lt;=$A$19,$D$19,IF(M143&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M143-INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M143,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y143">
-        <f>IF(M143="","",$B$5*TAN(RADIANS(M143))*(1+X143/100)*1000/$B$4)</f>
+        <f>IF(X143="","",X143*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12569,11 +12569,11 @@
         <v/>
       </c>
       <c r="X144">
-        <f>IF(OR($E$13&lt;&gt;"OK",M144=""),"",IF(M144&lt;=$A$19,$B$19,IF(M144&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M144-INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M144=""),"",IF(M144&lt;=$A$19,$D$19,IF(M144&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M144-INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M144,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y144">
-        <f>IF(M144="","",$B$5*TAN(RADIANS(M144))*(1+X144/100)*1000/$B$4)</f>
+        <f>IF(X144="","",X144*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12661,11 +12661,11 @@
         <v/>
       </c>
       <c r="X145">
-        <f>IF(OR($E$13&lt;&gt;"OK",M145=""),"",IF(M145&lt;=$A$19,$B$19,IF(M145&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M145-INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M145=""),"",IF(M145&lt;=$A$19,$D$19,IF(M145&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M145-INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M145,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y145">
-        <f>IF(M145="","",$B$5*TAN(RADIANS(M145))*(1+X145/100)*1000/$B$4)</f>
+        <f>IF(X145="","",X145*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12753,11 +12753,11 @@
         <v/>
       </c>
       <c r="X146">
-        <f>IF(OR($E$13&lt;&gt;"OK",M146=""),"",IF(M146&lt;=$A$19,$B$19,IF(M146&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M146-INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M146=""),"",IF(M146&lt;=$A$19,$D$19,IF(M146&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M146-INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M146,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y146">
-        <f>IF(M146="","",$B$5*TAN(RADIANS(M146))*(1+X146/100)*1000/$B$4)</f>
+        <f>IF(X146="","",X146*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12845,11 +12845,11 @@
         <v/>
       </c>
       <c r="X147">
-        <f>IF(OR($E$13&lt;&gt;"OK",M147=""),"",IF(M147&lt;=$A$19,$B$19,IF(M147&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M147-INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M147=""),"",IF(M147&lt;=$A$19,$D$19,IF(M147&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M147-INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M147,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y147">
-        <f>IF(M147="","",$B$5*TAN(RADIANS(M147))*(1+X147/100)*1000/$B$4)</f>
+        <f>IF(X147="","",X147*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -12937,11 +12937,11 @@
         <v/>
       </c>
       <c r="X148">
-        <f>IF(OR($E$13&lt;&gt;"OK",M148=""),"",IF(M148&lt;=$A$19,$B$19,IF(M148&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M148-INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M148=""),"",IF(M148&lt;=$A$19,$D$19,IF(M148&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M148-INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M148,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y148">
-        <f>IF(M148="","",$B$5*TAN(RADIANS(M148))*(1+X148/100)*1000/$B$4)</f>
+        <f>IF(X148="","",X148*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13029,11 +13029,11 @@
         <v/>
       </c>
       <c r="X149">
-        <f>IF(OR($E$13&lt;&gt;"OK",M149=""),"",IF(M149&lt;=$A$19,$B$19,IF(M149&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M149-INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M149=""),"",IF(M149&lt;=$A$19,$D$19,IF(M149&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M149-INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M149,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y149">
-        <f>IF(M149="","",$B$5*TAN(RADIANS(M149))*(1+X149/100)*1000/$B$4)</f>
+        <f>IF(X149="","",X149*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13121,11 +13121,11 @@
         <v/>
       </c>
       <c r="X150">
-        <f>IF(OR($E$13&lt;&gt;"OK",M150=""),"",IF(M150&lt;=$A$19,$B$19,IF(M150&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M150-INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M150=""),"",IF(M150&lt;=$A$19,$D$19,IF(M150&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M150-INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M150,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y150">
-        <f>IF(M150="","",$B$5*TAN(RADIANS(M150))*(1+X150/100)*1000/$B$4)</f>
+        <f>IF(X150="","",X150*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13213,11 +13213,11 @@
         <v/>
       </c>
       <c r="X151">
-        <f>IF(OR($E$13&lt;&gt;"OK",M151=""),"",IF(M151&lt;=$A$19,$B$19,IF(M151&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M151-INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M151=""),"",IF(M151&lt;=$A$19,$D$19,IF(M151&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M151-INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M151,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y151">
-        <f>IF(M151="","",$B$5*TAN(RADIANS(M151))*(1+X151/100)*1000/$B$4)</f>
+        <f>IF(X151="","",X151*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13305,11 +13305,11 @@
         <v/>
       </c>
       <c r="X152">
-        <f>IF(OR($E$13&lt;&gt;"OK",M152=""),"",IF(M152&lt;=$A$19,$B$19,IF(M152&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M152-INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M152=""),"",IF(M152&lt;=$A$19,$D$19,IF(M152&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M152-INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M152,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y152">
-        <f>IF(M152="","",$B$5*TAN(RADIANS(M152))*(1+X152/100)*1000/$B$4)</f>
+        <f>IF(X152="","",X152*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13397,11 +13397,11 @@
         <v/>
       </c>
       <c r="X153">
-        <f>IF(OR($E$13&lt;&gt;"OK",M153=""),"",IF(M153&lt;=$A$19,$B$19,IF(M153&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M153-INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M153=""),"",IF(M153&lt;=$A$19,$D$19,IF(M153&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M153-INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M153,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y153">
-        <f>IF(M153="","",$B$5*TAN(RADIANS(M153))*(1+X153/100)*1000/$B$4)</f>
+        <f>IF(X153="","",X153*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13489,11 +13489,11 @@
         <v/>
       </c>
       <c r="X154">
-        <f>IF(OR($E$13&lt;&gt;"OK",M154=""),"",IF(M154&lt;=$A$19,$B$19,IF(M154&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M154-INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M154=""),"",IF(M154&lt;=$A$19,$D$19,IF(M154&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M154-INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M154,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y154">
-        <f>IF(M154="","",$B$5*TAN(RADIANS(M154))*(1+X154/100)*1000/$B$4)</f>
+        <f>IF(X154="","",X154*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13581,11 +13581,11 @@
         <v/>
       </c>
       <c r="X155">
-        <f>IF(OR($E$13&lt;&gt;"OK",M155=""),"",IF(M155&lt;=$A$19,$B$19,IF(M155&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M155-INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M155=""),"",IF(M155&lt;=$A$19,$D$19,IF(M155&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M155-INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M155,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y155">
-        <f>IF(M155="","",$B$5*TAN(RADIANS(M155))*(1+X155/100)*1000/$B$4)</f>
+        <f>IF(X155="","",X155*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13673,11 +13673,11 @@
         <v/>
       </c>
       <c r="X156">
-        <f>IF(OR($E$13&lt;&gt;"OK",M156=""),"",IF(M156&lt;=$A$19,$B$19,IF(M156&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M156-INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M156=""),"",IF(M156&lt;=$A$19,$D$19,IF(M156&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M156-INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M156,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y156">
-        <f>IF(M156="","",$B$5*TAN(RADIANS(M156))*(1+X156/100)*1000/$B$4)</f>
+        <f>IF(X156="","",X156*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13765,11 +13765,11 @@
         <v/>
       </c>
       <c r="X157">
-        <f>IF(OR($E$13&lt;&gt;"OK",M157=""),"",IF(M157&lt;=$A$19,$B$19,IF(M157&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M157-INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M157=""),"",IF(M157&lt;=$A$19,$D$19,IF(M157&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M157-INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M157,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y157">
-        <f>IF(M157="","",$B$5*TAN(RADIANS(M157))*(1+X157/100)*1000/$B$4)</f>
+        <f>IF(X157="","",X157*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13857,11 +13857,11 @@
         <v/>
       </c>
       <c r="X158">
-        <f>IF(OR($E$13&lt;&gt;"OK",M158=""),"",IF(M158&lt;=$A$19,$B$19,IF(M158&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M158-INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M158=""),"",IF(M158&lt;=$A$19,$D$19,IF(M158&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M158-INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M158,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y158">
-        <f>IF(M158="","",$B$5*TAN(RADIANS(M158))*(1+X158/100)*1000/$B$4)</f>
+        <f>IF(X158="","",X158*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -13949,11 +13949,11 @@
         <v/>
       </c>
       <c r="X159">
-        <f>IF(OR($E$13&lt;&gt;"OK",M159=""),"",IF(M159&lt;=$A$19,$B$19,IF(M159&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M159-INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M159=""),"",IF(M159&lt;=$A$19,$D$19,IF(M159&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M159-INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M159,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y159">
-        <f>IF(M159="","",$B$5*TAN(RADIANS(M159))*(1+X159/100)*1000/$B$4)</f>
+        <f>IF(X159="","",X159*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14041,11 +14041,11 @@
         <v/>
       </c>
       <c r="X160">
-        <f>IF(OR($E$13&lt;&gt;"OK",M160=""),"",IF(M160&lt;=$A$19,$B$19,IF(M160&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M160-INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M160=""),"",IF(M160&lt;=$A$19,$D$19,IF(M160&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M160-INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M160,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y160">
-        <f>IF(M160="","",$B$5*TAN(RADIANS(M160))*(1+X160/100)*1000/$B$4)</f>
+        <f>IF(X160="","",X160*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14133,11 +14133,11 @@
         <v/>
       </c>
       <c r="X161">
-        <f>IF(OR($E$13&lt;&gt;"OK",M161=""),"",IF(M161&lt;=$A$19,$B$19,IF(M161&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M161-INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M161=""),"",IF(M161&lt;=$A$19,$D$19,IF(M161&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M161-INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M161,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y161">
-        <f>IF(M161="","",$B$5*TAN(RADIANS(M161))*(1+X161/100)*1000/$B$4)</f>
+        <f>IF(X161="","",X161*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14225,11 +14225,11 @@
         <v/>
       </c>
       <c r="X162">
-        <f>IF(OR($E$13&lt;&gt;"OK",M162=""),"",IF(M162&lt;=$A$19,$B$19,IF(M162&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M162-INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M162=""),"",IF(M162&lt;=$A$19,$D$19,IF(M162&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M162-INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M162,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y162">
-        <f>IF(M162="","",$B$5*TAN(RADIANS(M162))*(1+X162/100)*1000/$B$4)</f>
+        <f>IF(X162="","",X162*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14317,11 +14317,11 @@
         <v/>
       </c>
       <c r="X163">
-        <f>IF(OR($E$13&lt;&gt;"OK",M163=""),"",IF(M163&lt;=$A$19,$B$19,IF(M163&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M163-INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M163=""),"",IF(M163&lt;=$A$19,$D$19,IF(M163&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M163-INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M163,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y163">
-        <f>IF(M163="","",$B$5*TAN(RADIANS(M163))*(1+X163/100)*1000/$B$4)</f>
+        <f>IF(X163="","",X163*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14409,11 +14409,11 @@
         <v/>
       </c>
       <c r="X164">
-        <f>IF(OR($E$13&lt;&gt;"OK",M164=""),"",IF(M164&lt;=$A$19,$B$19,IF(M164&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M164-INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M164=""),"",IF(M164&lt;=$A$19,$D$19,IF(M164&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M164-INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M164,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y164">
-        <f>IF(M164="","",$B$5*TAN(RADIANS(M164))*(1+X164/100)*1000/$B$4)</f>
+        <f>IF(X164="","",X164*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14501,11 +14501,11 @@
         <v/>
       </c>
       <c r="X165">
-        <f>IF(OR($E$13&lt;&gt;"OK",M165=""),"",IF(M165&lt;=$A$19,$B$19,IF(M165&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M165-INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M165=""),"",IF(M165&lt;=$A$19,$D$19,IF(M165&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M165-INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M165,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y165">
-        <f>IF(M165="","",$B$5*TAN(RADIANS(M165))*(1+X165/100)*1000/$B$4)</f>
+        <f>IF(X165="","",X165*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14593,11 +14593,11 @@
         <v/>
       </c>
       <c r="X166">
-        <f>IF(OR($E$13&lt;&gt;"OK",M166=""),"",IF(M166&lt;=$A$19,$B$19,IF(M166&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M166-INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M166=""),"",IF(M166&lt;=$A$19,$D$19,IF(M166&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M166-INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M166,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y166">
-        <f>IF(M166="","",$B$5*TAN(RADIANS(M166))*(1+X166/100)*1000/$B$4)</f>
+        <f>IF(X166="","",X166*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14685,11 +14685,11 @@
         <v/>
       </c>
       <c r="X167">
-        <f>IF(OR($E$13&lt;&gt;"OK",M167=""),"",IF(M167&lt;=$A$19,$B$19,IF(M167&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M167-INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M167=""),"",IF(M167&lt;=$A$19,$D$19,IF(M167&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M167-INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M167,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y167">
-        <f>IF(M167="","",$B$5*TAN(RADIANS(M167))*(1+X167/100)*1000/$B$4)</f>
+        <f>IF(X167="","",X167*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14777,11 +14777,11 @@
         <v/>
       </c>
       <c r="X168">
-        <f>IF(OR($E$13&lt;&gt;"OK",M168=""),"",IF(M168&lt;=$A$19,$B$19,IF(M168&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M168-INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M168=""),"",IF(M168&lt;=$A$19,$D$19,IF(M168&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M168-INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M168,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y168">
-        <f>IF(M168="","",$B$5*TAN(RADIANS(M168))*(1+X168/100)*1000/$B$4)</f>
+        <f>IF(X168="","",X168*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14869,11 +14869,11 @@
         <v/>
       </c>
       <c r="X169">
-        <f>IF(OR($E$13&lt;&gt;"OK",M169=""),"",IF(M169&lt;=$A$19,$B$19,IF(M169&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M169-INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M169=""),"",IF(M169&lt;=$A$19,$D$19,IF(M169&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M169-INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M169,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y169">
-        <f>IF(M169="","",$B$5*TAN(RADIANS(M169))*(1+X169/100)*1000/$B$4)</f>
+        <f>IF(X169="","",X169*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -14961,11 +14961,11 @@
         <v/>
       </c>
       <c r="X170">
-        <f>IF(OR($E$13&lt;&gt;"OK",M170=""),"",IF(M170&lt;=$A$19,$B$19,IF(M170&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M170-INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M170=""),"",IF(M170&lt;=$A$19,$D$19,IF(M170&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M170-INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M170,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y170">
-        <f>IF(M170="","",$B$5*TAN(RADIANS(M170))*(1+X170/100)*1000/$B$4)</f>
+        <f>IF(X170="","",X170*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15053,11 +15053,11 @@
         <v/>
       </c>
       <c r="X171">
-        <f>IF(OR($E$13&lt;&gt;"OK",M171=""),"",IF(M171&lt;=$A$19,$B$19,IF(M171&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M171-INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M171=""),"",IF(M171&lt;=$A$19,$D$19,IF(M171&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M171-INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M171,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y171">
-        <f>IF(M171="","",$B$5*TAN(RADIANS(M171))*(1+X171/100)*1000/$B$4)</f>
+        <f>IF(X171="","",X171*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15145,11 +15145,11 @@
         <v/>
       </c>
       <c r="X172">
-        <f>IF(OR($E$13&lt;&gt;"OK",M172=""),"",IF(M172&lt;=$A$19,$B$19,IF(M172&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M172-INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M172=""),"",IF(M172&lt;=$A$19,$D$19,IF(M172&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M172-INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M172,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y172">
-        <f>IF(M172="","",$B$5*TAN(RADIANS(M172))*(1+X172/100)*1000/$B$4)</f>
+        <f>IF(X172="","",X172*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15237,11 +15237,11 @@
         <v/>
       </c>
       <c r="X173">
-        <f>IF(OR($E$13&lt;&gt;"OK",M173=""),"",IF(M173&lt;=$A$19,$B$19,IF(M173&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M173-INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M173=""),"",IF(M173&lt;=$A$19,$D$19,IF(M173&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M173-INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M173,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y173">
-        <f>IF(M173="","",$B$5*TAN(RADIANS(M173))*(1+X173/100)*1000/$B$4)</f>
+        <f>IF(X173="","",X173*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15329,11 +15329,11 @@
         <v/>
       </c>
       <c r="X174">
-        <f>IF(OR($E$13&lt;&gt;"OK",M174=""),"",IF(M174&lt;=$A$19,$B$19,IF(M174&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M174-INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M174=""),"",IF(M174&lt;=$A$19,$D$19,IF(M174&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M174-INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M174,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y174">
-        <f>IF(M174="","",$B$5*TAN(RADIANS(M174))*(1+X174/100)*1000/$B$4)</f>
+        <f>IF(X174="","",X174*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15421,11 +15421,11 @@
         <v/>
       </c>
       <c r="X175">
-        <f>IF(OR($E$13&lt;&gt;"OK",M175=""),"",IF(M175&lt;=$A$19,$B$19,IF(M175&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M175-INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M175=""),"",IF(M175&lt;=$A$19,$D$19,IF(M175&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M175-INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M175,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y175">
-        <f>IF(M175="","",$B$5*TAN(RADIANS(M175))*(1+X175/100)*1000/$B$4)</f>
+        <f>IF(X175="","",X175*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15513,11 +15513,11 @@
         <v/>
       </c>
       <c r="X176">
-        <f>IF(OR($E$13&lt;&gt;"OK",M176=""),"",IF(M176&lt;=$A$19,$B$19,IF(M176&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M176-INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M176=""),"",IF(M176&lt;=$A$19,$D$19,IF(M176&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M176-INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M176,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y176">
-        <f>IF(M176="","",$B$5*TAN(RADIANS(M176))*(1+X176/100)*1000/$B$4)</f>
+        <f>IF(X176="","",X176*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15605,11 +15605,11 @@
         <v/>
       </c>
       <c r="X177">
-        <f>IF(OR($E$13&lt;&gt;"OK",M177=""),"",IF(M177&lt;=$A$19,$B$19,IF(M177&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M177-INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M177=""),"",IF(M177&lt;=$A$19,$D$19,IF(M177&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M177-INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M177,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y177">
-        <f>IF(M177="","",$B$5*TAN(RADIANS(M177))*(1+X177/100)*1000/$B$4)</f>
+        <f>IF(X177="","",X177*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15697,11 +15697,11 @@
         <v/>
       </c>
       <c r="X178">
-        <f>IF(OR($E$13&lt;&gt;"OK",M178=""),"",IF(M178&lt;=$A$19,$B$19,IF(M178&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M178-INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M178=""),"",IF(M178&lt;=$A$19,$D$19,IF(M178&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M178-INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M178,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y178">
-        <f>IF(M178="","",$B$5*TAN(RADIANS(M178))*(1+X178/100)*1000/$B$4)</f>
+        <f>IF(X178="","",X178*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15789,11 +15789,11 @@
         <v/>
       </c>
       <c r="X179">
-        <f>IF(OR($E$13&lt;&gt;"OK",M179=""),"",IF(M179&lt;=$A$19,$B$19,IF(M179&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M179-INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M179=""),"",IF(M179&lt;=$A$19,$D$19,IF(M179&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M179-INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M179,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y179">
-        <f>IF(M179="","",$B$5*TAN(RADIANS(M179))*(1+X179/100)*1000/$B$4)</f>
+        <f>IF(X179="","",X179*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15881,11 +15881,11 @@
         <v/>
       </c>
       <c r="X180">
-        <f>IF(OR($E$13&lt;&gt;"OK",M180=""),"",IF(M180&lt;=$A$19,$B$19,IF(M180&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M180-INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M180=""),"",IF(M180&lt;=$A$19,$D$19,IF(M180&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M180-INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M180,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y180">
-        <f>IF(M180="","",$B$5*TAN(RADIANS(M180))*(1+X180/100)*1000/$B$4)</f>
+        <f>IF(X180="","",X180*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -15973,11 +15973,11 @@
         <v/>
       </c>
       <c r="X181">
-        <f>IF(OR($E$13&lt;&gt;"OK",M181=""),"",IF(M181&lt;=$A$19,$B$19,IF(M181&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M181-INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M181=""),"",IF(M181&lt;=$A$19,$D$19,IF(M181&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M181-INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M181,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y181">
-        <f>IF(M181="","",$B$5*TAN(RADIANS(M181))*(1+X181/100)*1000/$B$4)</f>
+        <f>IF(X181="","",X181*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16065,11 +16065,11 @@
         <v/>
       </c>
       <c r="X182">
-        <f>IF(OR($E$13&lt;&gt;"OK",M182=""),"",IF(M182&lt;=$A$19,$B$19,IF(M182&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M182-INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M182=""),"",IF(M182&lt;=$A$19,$D$19,IF(M182&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M182-INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M182,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y182">
-        <f>IF(M182="","",$B$5*TAN(RADIANS(M182))*(1+X182/100)*1000/$B$4)</f>
+        <f>IF(X182="","",X182*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16157,11 +16157,11 @@
         <v/>
       </c>
       <c r="X183">
-        <f>IF(OR($E$13&lt;&gt;"OK",M183=""),"",IF(M183&lt;=$A$19,$B$19,IF(M183&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M183-INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M183=""),"",IF(M183&lt;=$A$19,$D$19,IF(M183&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M183-INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M183,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y183">
-        <f>IF(M183="","",$B$5*TAN(RADIANS(M183))*(1+X183/100)*1000/$B$4)</f>
+        <f>IF(X183="","",X183*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16249,11 +16249,11 @@
         <v/>
       </c>
       <c r="X184">
-        <f>IF(OR($E$13&lt;&gt;"OK",M184=""),"",IF(M184&lt;=$A$19,$B$19,IF(M184&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M184-INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M184=""),"",IF(M184&lt;=$A$19,$D$19,IF(M184&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M184-INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M184,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y184">
-        <f>IF(M184="","",$B$5*TAN(RADIANS(M184))*(1+X184/100)*1000/$B$4)</f>
+        <f>IF(X184="","",X184*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16341,11 +16341,11 @@
         <v/>
       </c>
       <c r="X185">
-        <f>IF(OR($E$13&lt;&gt;"OK",M185=""),"",IF(M185&lt;=$A$19,$B$19,IF(M185&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M185-INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M185=""),"",IF(M185&lt;=$A$19,$D$19,IF(M185&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M185-INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M185,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y185">
-        <f>IF(M185="","",$B$5*TAN(RADIANS(M185))*(1+X185/100)*1000/$B$4)</f>
+        <f>IF(X185="","",X185*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16433,11 +16433,11 @@
         <v/>
       </c>
       <c r="X186">
-        <f>IF(OR($E$13&lt;&gt;"OK",M186=""),"",IF(M186&lt;=$A$19,$B$19,IF(M186&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M186-INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M186=""),"",IF(M186&lt;=$A$19,$D$19,IF(M186&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M186-INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M186,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y186">
-        <f>IF(M186="","",$B$5*TAN(RADIANS(M186))*(1+X186/100)*1000/$B$4)</f>
+        <f>IF(X186="","",X186*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16525,11 +16525,11 @@
         <v/>
       </c>
       <c r="X187">
-        <f>IF(OR($E$13&lt;&gt;"OK",M187=""),"",IF(M187&lt;=$A$19,$B$19,IF(M187&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M187-INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M187=""),"",IF(M187&lt;=$A$19,$D$19,IF(M187&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M187-INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M187,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y187">
-        <f>IF(M187="","",$B$5*TAN(RADIANS(M187))*(1+X187/100)*1000/$B$4)</f>
+        <f>IF(X187="","",X187*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16617,11 +16617,11 @@
         <v/>
       </c>
       <c r="X188">
-        <f>IF(OR($E$13&lt;&gt;"OK",M188=""),"",IF(M188&lt;=$A$19,$B$19,IF(M188&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M188-INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M188=""),"",IF(M188&lt;=$A$19,$D$19,IF(M188&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M188-INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M188,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y188">
-        <f>IF(M188="","",$B$5*TAN(RADIANS(M188))*(1+X188/100)*1000/$B$4)</f>
+        <f>IF(X188="","",X188*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16709,11 +16709,11 @@
         <v/>
       </c>
       <c r="X189">
-        <f>IF(OR($E$13&lt;&gt;"OK",M189=""),"",IF(M189&lt;=$A$19,$B$19,IF(M189&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M189-INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M189=""),"",IF(M189&lt;=$A$19,$D$19,IF(M189&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M189-INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M189,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y189">
-        <f>IF(M189="","",$B$5*TAN(RADIANS(M189))*(1+X189/100)*1000/$B$4)</f>
+        <f>IF(X189="","",X189*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16801,11 +16801,11 @@
         <v/>
       </c>
       <c r="X190">
-        <f>IF(OR($E$13&lt;&gt;"OK",M190=""),"",IF(M190&lt;=$A$19,$B$19,IF(M190&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M190-INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M190=""),"",IF(M190&lt;=$A$19,$D$19,IF(M190&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M190-INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M190,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y190">
-        <f>IF(M190="","",$B$5*TAN(RADIANS(M190))*(1+X190/100)*1000/$B$4)</f>
+        <f>IF(X190="","",X190*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16893,11 +16893,11 @@
         <v/>
       </c>
       <c r="X191">
-        <f>IF(OR($E$13&lt;&gt;"OK",M191=""),"",IF(M191&lt;=$A$19,$B$19,IF(M191&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M191-INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M191=""),"",IF(M191&lt;=$A$19,$D$19,IF(M191&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M191-INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M191,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y191">
-        <f>IF(M191="","",$B$5*TAN(RADIANS(M191))*(1+X191/100)*1000/$B$4)</f>
+        <f>IF(X191="","",X191*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -16985,11 +16985,11 @@
         <v/>
       </c>
       <c r="X192">
-        <f>IF(OR($E$13&lt;&gt;"OK",M192=""),"",IF(M192&lt;=$A$19,$B$19,IF(M192&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M192-INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M192=""),"",IF(M192&lt;=$A$19,$D$19,IF(M192&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M192-INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M192,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y192">
-        <f>IF(M192="","",$B$5*TAN(RADIANS(M192))*(1+X192/100)*1000/$B$4)</f>
+        <f>IF(X192="","",X192*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17077,11 +17077,11 @@
         <v/>
       </c>
       <c r="X193">
-        <f>IF(OR($E$13&lt;&gt;"OK",M193=""),"",IF(M193&lt;=$A$19,$B$19,IF(M193&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M193-INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M193=""),"",IF(M193&lt;=$A$19,$D$19,IF(M193&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M193-INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M193,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y193">
-        <f>IF(M193="","",$B$5*TAN(RADIANS(M193))*(1+X193/100)*1000/$B$4)</f>
+        <f>IF(X193="","",X193*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17169,11 +17169,11 @@
         <v/>
       </c>
       <c r="X194">
-        <f>IF(OR($E$13&lt;&gt;"OK",M194=""),"",IF(M194&lt;=$A$19,$B$19,IF(M194&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M194-INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M194=""),"",IF(M194&lt;=$A$19,$D$19,IF(M194&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M194-INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M194,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y194">
-        <f>IF(M194="","",$B$5*TAN(RADIANS(M194))*(1+X194/100)*1000/$B$4)</f>
+        <f>IF(X194="","",X194*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17261,11 +17261,11 @@
         <v/>
       </c>
       <c r="X195">
-        <f>IF(OR($E$13&lt;&gt;"OK",M195=""),"",IF(M195&lt;=$A$19,$B$19,IF(M195&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M195-INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M195=""),"",IF(M195&lt;=$A$19,$D$19,IF(M195&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M195-INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M195,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y195">
-        <f>IF(M195="","",$B$5*TAN(RADIANS(M195))*(1+X195/100)*1000/$B$4)</f>
+        <f>IF(X195="","",X195*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17353,11 +17353,11 @@
         <v/>
       </c>
       <c r="X196">
-        <f>IF(OR($E$13&lt;&gt;"OK",M196=""),"",IF(M196&lt;=$A$19,$B$19,IF(M196&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M196-INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M196=""),"",IF(M196&lt;=$A$19,$D$19,IF(M196&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M196-INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M196,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y196">
-        <f>IF(M196="","",$B$5*TAN(RADIANS(M196))*(1+X196/100)*1000/$B$4)</f>
+        <f>IF(X196="","",X196*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17445,11 +17445,11 @@
         <v/>
       </c>
       <c r="X197">
-        <f>IF(OR($E$13&lt;&gt;"OK",M197=""),"",IF(M197&lt;=$A$19,$B$19,IF(M197&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M197-INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M197=""),"",IF(M197&lt;=$A$19,$D$19,IF(M197&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M197-INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M197,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y197">
-        <f>IF(M197="","",$B$5*TAN(RADIANS(M197))*(1+X197/100)*1000/$B$4)</f>
+        <f>IF(X197="","",X197*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17537,11 +17537,11 @@
         <v/>
       </c>
       <c r="X198">
-        <f>IF(OR($E$13&lt;&gt;"OK",M198=""),"",IF(M198&lt;=$A$19,$B$19,IF(M198&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M198-INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M198=""),"",IF(M198&lt;=$A$19,$D$19,IF(M198&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M198-INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M198,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y198">
-        <f>IF(M198="","",$B$5*TAN(RADIANS(M198))*(1+X198/100)*1000/$B$4)</f>
+        <f>IF(X198="","",X198*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17629,11 +17629,11 @@
         <v/>
       </c>
       <c r="X199">
-        <f>IF(OR($E$13&lt;&gt;"OK",M199=""),"",IF(M199&lt;=$A$19,$B$19,IF(M199&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M199-INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M199=""),"",IF(M199&lt;=$A$19,$D$19,IF(M199&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M199-INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M199,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y199">
-        <f>IF(M199="","",$B$5*TAN(RADIANS(M199))*(1+X199/100)*1000/$B$4)</f>
+        <f>IF(X199="","",X199*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17721,11 +17721,11 @@
         <v/>
       </c>
       <c r="X200">
-        <f>IF(OR($E$13&lt;&gt;"OK",M200=""),"",IF(M200&lt;=$A$19,$B$19,IF(M200&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M200-INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M200=""),"",IF(M200&lt;=$A$19,$D$19,IF(M200&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M200-INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M200,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y200">
-        <f>IF(M200="","",$B$5*TAN(RADIANS(M200))*(1+X200/100)*1000/$B$4)</f>
+        <f>IF(X200="","",X200*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17813,11 +17813,11 @@
         <v/>
       </c>
       <c r="X201">
-        <f>IF(OR($E$13&lt;&gt;"OK",M201=""),"",IF(M201&lt;=$A$19,$B$19,IF(M201&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M201-INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M201=""),"",IF(M201&lt;=$A$19,$D$19,IF(M201&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M201-INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M201,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y201">
-        <f>IF(M201="","",$B$5*TAN(RADIANS(M201))*(1+X201/100)*1000/$B$4)</f>
+        <f>IF(X201="","",X201*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17905,11 +17905,11 @@
         <v/>
       </c>
       <c r="X202">
-        <f>IF(OR($E$13&lt;&gt;"OK",M202=""),"",IF(M202&lt;=$A$19,$B$19,IF(M202&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M202-INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M202=""),"",IF(M202&lt;=$A$19,$D$19,IF(M202&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M202-INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M202,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y202">
-        <f>IF(M202="","",$B$5*TAN(RADIANS(M202))*(1+X202/100)*1000/$B$4)</f>
+        <f>IF(X202="","",X202*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -17997,11 +17997,11 @@
         <v/>
       </c>
       <c r="X203">
-        <f>IF(OR($E$13&lt;&gt;"OK",M203=""),"",IF(M203&lt;=$A$19,$B$19,IF(M203&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M203-INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M203=""),"",IF(M203&lt;=$A$19,$D$19,IF(M203&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M203-INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M203,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y203">
-        <f>IF(M203="","",$B$5*TAN(RADIANS(M203))*(1+X203/100)*1000/$B$4)</f>
+        <f>IF(X203="","",X203*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18089,11 +18089,11 @@
         <v/>
       </c>
       <c r="X204">
-        <f>IF(OR($E$13&lt;&gt;"OK",M204=""),"",IF(M204&lt;=$A$19,$B$19,IF(M204&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M204-INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M204=""),"",IF(M204&lt;=$A$19,$D$19,IF(M204&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M204-INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M204,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y204">
-        <f>IF(M204="","",$B$5*TAN(RADIANS(M204))*(1+X204/100)*1000/$B$4)</f>
+        <f>IF(X204="","",X204*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18181,11 +18181,11 @@
         <v/>
       </c>
       <c r="X205">
-        <f>IF(OR($E$13&lt;&gt;"OK",M205=""),"",IF(M205&lt;=$A$19,$B$19,IF(M205&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M205-INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M205=""),"",IF(M205&lt;=$A$19,$D$19,IF(M205&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M205-INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M205,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y205">
-        <f>IF(M205="","",$B$5*TAN(RADIANS(M205))*(1+X205/100)*1000/$B$4)</f>
+        <f>IF(X205="","",X205*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18273,11 +18273,11 @@
         <v/>
       </c>
       <c r="X206">
-        <f>IF(OR($E$13&lt;&gt;"OK",M206=""),"",IF(M206&lt;=$A$19,$B$19,IF(M206&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M206-INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M206=""),"",IF(M206&lt;=$A$19,$D$19,IF(M206&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M206-INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M206,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y206">
-        <f>IF(M206="","",$B$5*TAN(RADIANS(M206))*(1+X206/100)*1000/$B$4)</f>
+        <f>IF(X206="","",X206*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18365,11 +18365,11 @@
         <v/>
       </c>
       <c r="X207">
-        <f>IF(OR($E$13&lt;&gt;"OK",M207=""),"",IF(M207&lt;=$A$19,$B$19,IF(M207&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M207-INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M207=""),"",IF(M207&lt;=$A$19,$D$19,IF(M207&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M207-INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M207,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y207">
-        <f>IF(M207="","",$B$5*TAN(RADIANS(M207))*(1+X207/100)*1000/$B$4)</f>
+        <f>IF(X207="","",X207*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18457,11 +18457,11 @@
         <v/>
       </c>
       <c r="X208">
-        <f>IF(OR($E$13&lt;&gt;"OK",M208=""),"",IF(M208&lt;=$A$19,$B$19,IF(M208&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M208-INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M208=""),"",IF(M208&lt;=$A$19,$D$19,IF(M208&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M208-INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M208,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y208">
-        <f>IF(M208="","",$B$5*TAN(RADIANS(M208))*(1+X208/100)*1000/$B$4)</f>
+        <f>IF(X208="","",X208*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18549,11 +18549,11 @@
         <v/>
       </c>
       <c r="X209">
-        <f>IF(OR($E$13&lt;&gt;"OK",M209=""),"",IF(M209&lt;=$A$19,$B$19,IF(M209&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M209-INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M209=""),"",IF(M209&lt;=$A$19,$D$19,IF(M209&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M209-INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M209,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y209">
-        <f>IF(M209="","",$B$5*TAN(RADIANS(M209))*(1+X209/100)*1000/$B$4)</f>
+        <f>IF(X209="","",X209*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18641,11 +18641,11 @@
         <v/>
       </c>
       <c r="X210">
-        <f>IF(OR($E$13&lt;&gt;"OK",M210=""),"",IF(M210&lt;=$A$19,$B$19,IF(M210&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M210-INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M210=""),"",IF(M210&lt;=$A$19,$D$19,IF(M210&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M210-INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M210,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y210">
-        <f>IF(M210="","",$B$5*TAN(RADIANS(M210))*(1+X210/100)*1000/$B$4)</f>
+        <f>IF(X210="","",X210*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18733,11 +18733,11 @@
         <v/>
       </c>
       <c r="X211">
-        <f>IF(OR($E$13&lt;&gt;"OK",M211=""),"",IF(M211&lt;=$A$19,$B$19,IF(M211&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M211-INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M211=""),"",IF(M211&lt;=$A$19,$D$19,IF(M211&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M211-INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M211,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y211">
-        <f>IF(M211="","",$B$5*TAN(RADIANS(M211))*(1+X211/100)*1000/$B$4)</f>
+        <f>IF(X211="","",X211*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18825,11 +18825,11 @@
         <v/>
       </c>
       <c r="X212">
-        <f>IF(OR($E$13&lt;&gt;"OK",M212=""),"",IF(M212&lt;=$A$19,$B$19,IF(M212&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M212-INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M212=""),"",IF(M212&lt;=$A$19,$D$19,IF(M212&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M212-INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M212,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y212">
-        <f>IF(M212="","",$B$5*TAN(RADIANS(M212))*(1+X212/100)*1000/$B$4)</f>
+        <f>IF(X212="","",X212*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -18917,11 +18917,11 @@
         <v/>
       </c>
       <c r="X213">
-        <f>IF(OR($E$13&lt;&gt;"OK",M213=""),"",IF(M213&lt;=$A$19,$B$19,IF(M213&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M213-INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M213=""),"",IF(M213&lt;=$A$19,$D$19,IF(M213&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M213-INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M213,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y213">
-        <f>IF(M213="","",$B$5*TAN(RADIANS(M213))*(1+X213/100)*1000/$B$4)</f>
+        <f>IF(X213="","",X213*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19009,11 +19009,11 @@
         <v/>
       </c>
       <c r="X214">
-        <f>IF(OR($E$13&lt;&gt;"OK",M214=""),"",IF(M214&lt;=$A$19,$B$19,IF(M214&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M214-INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M214=""),"",IF(M214&lt;=$A$19,$D$19,IF(M214&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M214-INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M214,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y214">
-        <f>IF(M214="","",$B$5*TAN(RADIANS(M214))*(1+X214/100)*1000/$B$4)</f>
+        <f>IF(X214="","",X214*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19101,11 +19101,11 @@
         <v/>
       </c>
       <c r="X215">
-        <f>IF(OR($E$13&lt;&gt;"OK",M215=""),"",IF(M215&lt;=$A$19,$B$19,IF(M215&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M215-INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M215=""),"",IF(M215&lt;=$A$19,$D$19,IF(M215&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M215-INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M215,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y215">
-        <f>IF(M215="","",$B$5*TAN(RADIANS(M215))*(1+X215/100)*1000/$B$4)</f>
+        <f>IF(X215="","",X215*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19193,11 +19193,11 @@
         <v/>
       </c>
       <c r="X216">
-        <f>IF(OR($E$13&lt;&gt;"OK",M216=""),"",IF(M216&lt;=$A$19,$B$19,IF(M216&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M216-INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M216=""),"",IF(M216&lt;=$A$19,$D$19,IF(M216&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M216-INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M216,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y216">
-        <f>IF(M216="","",$B$5*TAN(RADIANS(M216))*(1+X216/100)*1000/$B$4)</f>
+        <f>IF(X216="","",X216*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19285,11 +19285,11 @@
         <v/>
       </c>
       <c r="X217">
-        <f>IF(OR($E$13&lt;&gt;"OK",M217=""),"",IF(M217&lt;=$A$19,$B$19,IF(M217&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M217-INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M217=""),"",IF(M217&lt;=$A$19,$D$19,IF(M217&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M217-INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M217,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y217">
-        <f>IF(M217="","",$B$5*TAN(RADIANS(M217))*(1+X217/100)*1000/$B$4)</f>
+        <f>IF(X217="","",X217*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19377,11 +19377,11 @@
         <v/>
       </c>
       <c r="X218">
-        <f>IF(OR($E$13&lt;&gt;"OK",M218=""),"",IF(M218&lt;=$A$19,$B$19,IF(M218&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M218-INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M218=""),"",IF(M218&lt;=$A$19,$D$19,IF(M218&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M218-INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M218,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y218">
-        <f>IF(M218="","",$B$5*TAN(RADIANS(M218))*(1+X218/100)*1000/$B$4)</f>
+        <f>IF(X218="","",X218*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19455,11 +19455,11 @@
         <v/>
       </c>
       <c r="X219">
-        <f>IF(OR($E$13&lt;&gt;"OK",M219=""),"",IF(M219&lt;=$A$19,$B$19,IF(M219&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M219-INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M219=""),"",IF(M219&lt;=$A$19,$D$19,IF(M219&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M219-INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M219,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y219">
-        <f>IF(M219="","",$B$5*TAN(RADIANS(M219))*(1+X219/100)*1000/$B$4)</f>
+        <f>IF(X219="","",X219*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19533,11 +19533,11 @@
         <v/>
       </c>
       <c r="X220">
-        <f>IF(OR($E$13&lt;&gt;"OK",M220=""),"",IF(M220&lt;=$A$19,$B$19,IF(M220&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M220-INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M220=""),"",IF(M220&lt;=$A$19,$D$19,IF(M220&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M220-INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M220,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y220">
-        <f>IF(M220="","",$B$5*TAN(RADIANS(M220))*(1+X220/100)*1000/$B$4)</f>
+        <f>IF(X220="","",X220*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19611,11 +19611,11 @@
         <v/>
       </c>
       <c r="X221">
-        <f>IF(OR($E$13&lt;&gt;"OK",M221=""),"",IF(M221&lt;=$A$19,$B$19,IF(M221&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M221-INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M221=""),"",IF(M221&lt;=$A$19,$D$19,IF(M221&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M221-INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M221,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y221">
-        <f>IF(M221="","",$B$5*TAN(RADIANS(M221))*(1+X221/100)*1000/$B$4)</f>
+        <f>IF(X221="","",X221*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19689,11 +19689,11 @@
         <v/>
       </c>
       <c r="X222">
-        <f>IF(OR($E$13&lt;&gt;"OK",M222=""),"",IF(M222&lt;=$A$19,$B$19,IF(M222&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M222-INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M222=""),"",IF(M222&lt;=$A$19,$D$19,IF(M222&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M222-INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M222,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y222">
-        <f>IF(M222="","",$B$5*TAN(RADIANS(M222))*(1+X222/100)*1000/$B$4)</f>
+        <f>IF(X222="","",X222*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19767,11 +19767,11 @@
         <v/>
       </c>
       <c r="X223">
-        <f>IF(OR($E$13&lt;&gt;"OK",M223=""),"",IF(M223&lt;=$A$19,$B$19,IF(M223&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M223-INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M223=""),"",IF(M223&lt;=$A$19,$D$19,IF(M223&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M223-INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M223,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y223">
-        <f>IF(M223="","",$B$5*TAN(RADIANS(M223))*(1+X223/100)*1000/$B$4)</f>
+        <f>IF(X223="","",X223*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19845,11 +19845,11 @@
         <v/>
       </c>
       <c r="X224">
-        <f>IF(OR($E$13&lt;&gt;"OK",M224=""),"",IF(M224&lt;=$A$19,$B$19,IF(M224&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M224-INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M224=""),"",IF(M224&lt;=$A$19,$D$19,IF(M224&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M224-INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M224,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y224">
-        <f>IF(M224="","",$B$5*TAN(RADIANS(M224))*(1+X224/100)*1000/$B$4)</f>
+        <f>IF(X224="","",X224*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -19923,11 +19923,11 @@
         <v/>
       </c>
       <c r="X225">
-        <f>IF(OR($E$13&lt;&gt;"OK",M225=""),"",IF(M225&lt;=$A$19,$B$19,IF(M225&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M225-INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M225=""),"",IF(M225&lt;=$A$19,$D$19,IF(M225&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M225-INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M225,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y225">
-        <f>IF(M225="","",$B$5*TAN(RADIANS(M225))*(1+X225/100)*1000/$B$4)</f>
+        <f>IF(X225="","",X225*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -20001,11 +20001,11 @@
         <v/>
       </c>
       <c r="X226">
-        <f>IF(OR($E$13&lt;&gt;"OK",M226=""),"",IF(M226&lt;=$A$19,$B$19,IF(M226&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M226-INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M226=""),"",IF(M226&lt;=$A$19,$D$19,IF(M226&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M226-INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M226,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y226">
-        <f>IF(M226="","",$B$5*TAN(RADIANS(M226))*(1+X226/100)*1000/$B$4)</f>
+        <f>IF(X226="","",X226*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -20079,11 +20079,11 @@
         <v/>
       </c>
       <c r="X227">
-        <f>IF(OR($E$13&lt;&gt;"OK",M227=""),"",IF(M227&lt;=$A$19,$B$19,IF(M227&gt;=INDEX($A$19:$A$218,$E$12),INDEX($B$19:$B$218,$E$12),INDEX($B$19:$B$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M227-INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($B$19:$B$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($B$19:$B$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
+        <f>IF(OR($E$13&lt;&gt;"OK",M227=""),"",IF(M227&lt;=$A$19,$D$19,IF(M227&gt;=INDEX($A$19:$A$218,$E$12),INDEX($D$19:$D$218,$E$12),INDEX($D$19:$D$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1))+(M227-INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)))*(INDEX($D$19:$D$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($D$19:$D$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)))/(INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1)+1)-INDEX($A$19:$A$218,MATCH(M227,$A$19:INDEX($A$19:$A$218,$E$12),1))))))</f>
         <v/>
       </c>
       <c r="Y227">
-        <f>IF(M227="","",$B$5*TAN(RADIANS(M227))*(1+X227/100)*1000/$B$4)</f>
+        <f>IF(X227="","",X227*1000/$B$4)</f>
         <v/>
       </c>
     </row>
@@ -20186,7 +20186,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>先以目標 sensor 半徑反查「畸變 sensor 半徑」得到半視角，再用 R=Z·tan(θ) 求物方半徑。超出表格時使用端點角度，不外插；應避免出現警告。</t>
+          <t>由每筆半視角／Distortion 先建立「半視角 ↔ 畸變 sensor 半徑」LUT，並在相鄰資料點間做分段線性內插；再用 R=Z·tan(θ) 求物方半徑。首列半視角必須為 0；超出表格時使用端點角度，不外插。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arrange TV-line levels vertically by field
Co-authored-by: Higanbana-TW <Higanbana-TW@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lens_distortion_line_calculator.xlsx
+++ b/lens_distortion_line_calculator.xlsx
@@ -944,11 +944,11 @@
         <v/>
       </c>
       <c r="O4" s="8">
-        <f>O5-N5/2-MIN(L4,L5)-N4/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P4" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P5-M5/2-MIN(L4,L5)-M4/2</f>
         <v/>
       </c>
     </row>
@@ -1008,11 +1008,11 @@
         <v/>
       </c>
       <c r="O5" s="8">
-        <f>O6-N6/2-MIN(L5,L6)-N5/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P5" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P6-M6/2-MIN(L5,L6)-M5/2</f>
         <v/>
       </c>
     </row>
@@ -1072,11 +1072,11 @@
         <v/>
       </c>
       <c r="O6" s="8">
-        <f>O7-N7/2-MIN(L6,L7)-N6/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P6" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P7-M7/2-MIN(L6,L7)-M6/2</f>
         <v/>
       </c>
     </row>
@@ -1137,11 +1137,11 @@
         <v/>
       </c>
       <c r="O7" s="8">
-        <f>O8-N8/2-MIN(L7,L8)-N7/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P7" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P8-M8/2-MIN(L7,L8)-M7/2</f>
         <v/>
       </c>
     </row>
@@ -1189,11 +1189,11 @@
         <v/>
       </c>
       <c r="O8" s="8">
-        <f>O9-N9/2-MIN(L8,L9)-N8/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P8" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P9-M9/2-MIN(L8,L9)-M8/2</f>
         <v/>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
         <is>
           <t>第一象限位置：X 向右、Y 向上。
 指定 TV本的橫／豎線組合中心位於半對角線指定倍率。
-橫線組在左、豎線組在右；11 級由低至高向右排列。</t>
+橫線組在左、豎線組在右；11 級由上到下排列。</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1289,11 +1289,11 @@
         <v/>
       </c>
       <c r="O10" s="8">
-        <f>O9+N9/2+MIN(L9,L10)+N10/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P10" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P9+M9/2+MIN(L9,L10)+M10/2</f>
         <v/>
       </c>
     </row>
@@ -1318,11 +1318,11 @@
         <v/>
       </c>
       <c r="O11" s="8">
-        <f>O10+N10/2+MIN(L10,L11)+N11/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P11" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P10+M10/2+MIN(L10,L11)+M11/2</f>
         <v/>
       </c>
     </row>
@@ -1347,11 +1347,11 @@
         <v/>
       </c>
       <c r="O12" s="8">
-        <f>O11+N11/2+MIN(L11,L12)+N12/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P12" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P11+M11/2+MIN(L11,L12)+M12/2</f>
         <v/>
       </c>
     </row>
@@ -1376,11 +1376,11 @@
         <v/>
       </c>
       <c r="O13" s="8">
-        <f>O12+N12/2+MIN(L12,L13)+N13/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P13" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P12+M12/2+MIN(L12,L13)+M13/2</f>
         <v/>
       </c>
     </row>
@@ -1405,11 +1405,11 @@
         <v/>
       </c>
       <c r="O14" s="8">
-        <f>O13+N13/2+MIN(L13,L14)+N14/2</f>
+        <f>$B$7/2+$E$6*$B$7/2</f>
         <v/>
       </c>
       <c r="P14" s="8">
-        <f>$B$8/2-$E$6*$B$8/2</f>
+        <f>P13+M13/2+MIN(L13,L14)+M14/2</f>
         <v/>
       </c>
     </row>
@@ -65323,7 +65323,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>預設指定 1500 TV本、間隔 100 TV本，自動產生 1000～2000 TV本，共 11 級。相鄰圖樣的間隔採兩級中較細的線寬。</t>
+          <t>預設指定 1500 TV本、間隔 100 TV本，自動產生 1000～2000 TV本，共 11 級。11 級垂直排列：1000 TV本在上方較外場，2000 TV本在下方較內場；相鄰圖樣的間隔採兩級中較細的線寬。</t>
         </is>
       </c>
     </row>

</xml_diff>